<commit_message>
Separar registro de gastos manual y mejorar itinerario tipo calendario
Nueva pestana "Registro de Gastos" de carga manual (Nico anota los
gastos reales dia a dia), con totales por nucleo via SUMIF y una
seccion de deudas entre personas (Universal pagado por German, ligada
por formula a la Matriz Financiera). "Itinerario Flash" ahora incluye
horarios reales y un estado Confirmado/Por organizar por actividad.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019LrLKneXbkjTi7bzStorH9
</commit_message>
<xml_diff>
--- a/Presupuesto_Florida_2027_Nico.xlsx
+++ b/Presupuesto_Florida_2027_Nico.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="Dashboard y Reglas" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Matriz Financiera" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Itinerario Flash" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Logistica Terrestre y Vuelos" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Guia Operativa" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Registro de Gastos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Itinerario Flash" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Logistica Terrestre y Vuelos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Guia Operativa" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="N1_PAX">'Matriz Financiera'!$J$2</definedName>
@@ -33,7 +34,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,6 +86,20 @@
     </font>
     <font>
       <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007F6000"/>
       <sz val="9.5"/>
     </font>
     <font>
@@ -97,7 +112,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -142,6 +157,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -215,7 +235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -274,32 +294,45 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="10" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -717,7 +750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -905,33 +938,40 @@
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>• Pestana 2 (Matriz Financiera): todas las celdas de costo total y costo de Nicolas son FORMULAS activas de Excel. Las celdas resaltadas en amarillo son estimaciones editables.</t>
+          <t>• Pestana 2 (Matriz Financiera): presupuesto PROYECTADO segun lo ya reservado/facturado. Todas las celdas de costo total y costo de Nicolas son FORMULAS activas de Excel. Las celdas resaltadas en amarillo son estimaciones editables.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>• Pestana 3 (Itinerario Flash): cruce dia a dia de actividades con los horarios reales de vuelo.</t>
+          <t>• Pestana 3 (Registro de Gastos): hoja de carga MANUAL para que Nico anote los gastos reales dia a dia (Uber, comidas, compras, etc.). Los totales por nucleo se calculan solos con formulas.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="26" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>• Pestana 4 (Logistica): tabla de vuelos reales (PNR ETPWSR / booking B4ZHG8) y analisis de alquiler de minivan en Miami.</t>
+          <t>• Pestana 4 (Itinerario Flash): calendario dia a dia con horarios reales de vuelo y estado Confirmado / Por organizar de cada actividad.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="26" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>• Pestana 5 (Guia Operativa): tips practicos y la formula de control del presupuesto total del grupo.</t>
+          <t>• Pestana 5 (Logistica): tabla de vuelos reales (PNR ETPWSR / booking B4ZHG8) y analisis de alquiler de minivan en Miami.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>• Pestana 6 (Guia Operativa): tips practicos y la formula de control del presupuesto total del grupo.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="C8:F8"/>
     <mergeCell ref="C7:F7"/>
@@ -949,6 +989,7 @@
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="C10:F10"/>
     <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="C9:F9"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -1427,64 +1468,958 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ITINERARIO FLASH - FEBRERO 2027</t>
+          <t>REGISTRO DE GASTOS - CARGA MANUAL (NICO)</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Esta hoja es de uso exclusivo de Nico: anotar aca cada gasto real a medida que ocurre en el viaje (Uber, comidas, compras, propinas, etc.). Es independiente de la Matriz Financiera (que refleja lo ya reservado/facturado). Los totales de abajo se recalculan solos con formulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B4" s="29" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="C4" s="29" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="D4" s="29" t="inlineStr">
+        <is>
+          <t>Nucleo</t>
+        </is>
+      </c>
+      <c r="E4" s="29" t="inlineStr">
+        <is>
+          <t>Pagado por</t>
+        </is>
+      </c>
+      <c r="F4" s="29" t="inlineStr">
+        <is>
+          <t>Monto USD</t>
+        </is>
+      </c>
+      <c r="G4" s="29" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="30" t="inlineStr">
+        <is>
+          <t>A confirmar</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="n"/>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>Sena de reserva (confirmar si es Universal 63W124U2 o Disney #43028783 - ambas por $200)</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="n"/>
+      <c r="E5" s="30" t="inlineStr">
+        <is>
+          <t>Nicolas - Tarjeta credito Santander Rio</t>
+        </is>
+      </c>
+      <c r="F5" s="32" t="n">
+        <v>200</v>
+      </c>
+      <c r="G5" s="30" t="inlineStr">
+        <is>
+          <t>Cargado por Claude a pedido de Nico; confirmar fecha exacta y a que reserva corresponde.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="33" t="n"/>
+      <c r="B6" s="33" t="n"/>
+      <c r="C6" s="33" t="n"/>
+      <c r="D6" s="33" t="n"/>
+      <c r="E6" s="33" t="n"/>
+      <c r="F6" s="34" t="n"/>
+      <c r="G6" s="33" t="n"/>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="31" t="n"/>
+      <c r="B7" s="31" t="n"/>
+      <c r="C7" s="31" t="n"/>
+      <c r="D7" s="31" t="n"/>
+      <c r="E7" s="31" t="n"/>
+      <c r="F7" s="32" t="n"/>
+      <c r="G7" s="31" t="n"/>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="33" t="n"/>
+      <c r="B8" s="33" t="n"/>
+      <c r="C8" s="33" t="n"/>
+      <c r="D8" s="33" t="n"/>
+      <c r="E8" s="33" t="n"/>
+      <c r="F8" s="34" t="n"/>
+      <c r="G8" s="33" t="n"/>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="31" t="n"/>
+      <c r="B9" s="31" t="n"/>
+      <c r="C9" s="31" t="n"/>
+      <c r="D9" s="31" t="n"/>
+      <c r="E9" s="31" t="n"/>
+      <c r="F9" s="32" t="n"/>
+      <c r="G9" s="31" t="n"/>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="33" t="n"/>
+      <c r="B10" s="33" t="n"/>
+      <c r="C10" s="33" t="n"/>
+      <c r="D10" s="33" t="n"/>
+      <c r="E10" s="33" t="n"/>
+      <c r="F10" s="34" t="n"/>
+      <c r="G10" s="33" t="n"/>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="31" t="n"/>
+      <c r="B11" s="31" t="n"/>
+      <c r="C11" s="31" t="n"/>
+      <c r="D11" s="31" t="n"/>
+      <c r="E11" s="31" t="n"/>
+      <c r="F11" s="32" t="n"/>
+      <c r="G11" s="31" t="n"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="33" t="n"/>
+      <c r="B12" s="33" t="n"/>
+      <c r="C12" s="33" t="n"/>
+      <c r="D12" s="33" t="n"/>
+      <c r="E12" s="33" t="n"/>
+      <c r="F12" s="34" t="n"/>
+      <c r="G12" s="33" t="n"/>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="31" t="n"/>
+      <c r="B13" s="31" t="n"/>
+      <c r="C13" s="31" t="n"/>
+      <c r="D13" s="31" t="n"/>
+      <c r="E13" s="31" t="n"/>
+      <c r="F13" s="32" t="n"/>
+      <c r="G13" s="31" t="n"/>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="33" t="n"/>
+      <c r="B14" s="33" t="n"/>
+      <c r="C14" s="33" t="n"/>
+      <c r="D14" s="33" t="n"/>
+      <c r="E14" s="33" t="n"/>
+      <c r="F14" s="34" t="n"/>
+      <c r="G14" s="33" t="n"/>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="31" t="n"/>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="31" t="n"/>
+      <c r="E15" s="31" t="n"/>
+      <c r="F15" s="32" t="n"/>
+      <c r="G15" s="31" t="n"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="33" t="n"/>
+      <c r="B16" s="33" t="n"/>
+      <c r="C16" s="33" t="n"/>
+      <c r="D16" s="33" t="n"/>
+      <c r="E16" s="33" t="n"/>
+      <c r="F16" s="34" t="n"/>
+      <c r="G16" s="33" t="n"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="31" t="n"/>
+      <c r="B17" s="31" t="n"/>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="31" t="n"/>
+      <c r="E17" s="31" t="n"/>
+      <c r="F17" s="32" t="n"/>
+      <c r="G17" s="31" t="n"/>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="33" t="n"/>
+      <c r="B18" s="33" t="n"/>
+      <c r="C18" s="33" t="n"/>
+      <c r="D18" s="33" t="n"/>
+      <c r="E18" s="33" t="n"/>
+      <c r="F18" s="34" t="n"/>
+      <c r="G18" s="33" t="n"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="31" t="n"/>
+      <c r="B19" s="31" t="n"/>
+      <c r="C19" s="31" t="n"/>
+      <c r="D19" s="31" t="n"/>
+      <c r="E19" s="31" t="n"/>
+      <c r="F19" s="32" t="n"/>
+      <c r="G19" s="31" t="n"/>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="33" t="n"/>
+      <c r="B20" s="33" t="n"/>
+      <c r="C20" s="33" t="n"/>
+      <c r="D20" s="33" t="n"/>
+      <c r="E20" s="33" t="n"/>
+      <c r="F20" s="34" t="n"/>
+      <c r="G20" s="33" t="n"/>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="31" t="n"/>
+      <c r="B21" s="31" t="n"/>
+      <c r="C21" s="31" t="n"/>
+      <c r="D21" s="31" t="n"/>
+      <c r="E21" s="31" t="n"/>
+      <c r="F21" s="32" t="n"/>
+      <c r="G21" s="31" t="n"/>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="33" t="n"/>
+      <c r="B22" s="33" t="n"/>
+      <c r="C22" s="33" t="n"/>
+      <c r="D22" s="33" t="n"/>
+      <c r="E22" s="33" t="n"/>
+      <c r="F22" s="34" t="n"/>
+      <c r="G22" s="33" t="n"/>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="31" t="n"/>
+      <c r="B23" s="31" t="n"/>
+      <c r="C23" s="31" t="n"/>
+      <c r="D23" s="31" t="n"/>
+      <c r="E23" s="31" t="n"/>
+      <c r="F23" s="32" t="n"/>
+      <c r="G23" s="31" t="n"/>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="33" t="n"/>
+      <c r="B24" s="33" t="n"/>
+      <c r="C24" s="33" t="n"/>
+      <c r="D24" s="33" t="n"/>
+      <c r="E24" s="33" t="n"/>
+      <c r="F24" s="34" t="n"/>
+      <c r="G24" s="33" t="n"/>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="31" t="n"/>
+      <c r="B25" s="31" t="n"/>
+      <c r="C25" s="31" t="n"/>
+      <c r="D25" s="31" t="n"/>
+      <c r="E25" s="31" t="n"/>
+      <c r="F25" s="32" t="n"/>
+      <c r="G25" s="31" t="n"/>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="33" t="n"/>
+      <c r="B26" s="33" t="n"/>
+      <c r="C26" s="33" t="n"/>
+      <c r="D26" s="33" t="n"/>
+      <c r="E26" s="33" t="n"/>
+      <c r="F26" s="34" t="n"/>
+      <c r="G26" s="33" t="n"/>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="31" t="n"/>
+      <c r="B27" s="31" t="n"/>
+      <c r="C27" s="31" t="n"/>
+      <c r="D27" s="31" t="n"/>
+      <c r="E27" s="31" t="n"/>
+      <c r="F27" s="32" t="n"/>
+      <c r="G27" s="31" t="n"/>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="33" t="n"/>
+      <c r="B28" s="33" t="n"/>
+      <c r="C28" s="33" t="n"/>
+      <c r="D28" s="33" t="n"/>
+      <c r="E28" s="33" t="n"/>
+      <c r="F28" s="34" t="n"/>
+      <c r="G28" s="33" t="n"/>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="31" t="n"/>
+      <c r="B29" s="31" t="n"/>
+      <c r="C29" s="31" t="n"/>
+      <c r="D29" s="31" t="n"/>
+      <c r="E29" s="31" t="n"/>
+      <c r="F29" s="32" t="n"/>
+      <c r="G29" s="31" t="n"/>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="33" t="n"/>
+      <c r="B30" s="33" t="n"/>
+      <c r="C30" s="33" t="n"/>
+      <c r="D30" s="33" t="n"/>
+      <c r="E30" s="33" t="n"/>
+      <c r="F30" s="34" t="n"/>
+      <c r="G30" s="33" t="n"/>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="31" t="n"/>
+      <c r="B31" s="31" t="n"/>
+      <c r="C31" s="31" t="n"/>
+      <c r="D31" s="31" t="n"/>
+      <c r="E31" s="31" t="n"/>
+      <c r="F31" s="32" t="n"/>
+      <c r="G31" s="31" t="n"/>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="33" t="n"/>
+      <c r="B32" s="33" t="n"/>
+      <c r="C32" s="33" t="n"/>
+      <c r="D32" s="33" t="n"/>
+      <c r="E32" s="33" t="n"/>
+      <c r="F32" s="34" t="n"/>
+      <c r="G32" s="33" t="n"/>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="31" t="n"/>
+      <c r="B33" s="31" t="n"/>
+      <c r="C33" s="31" t="n"/>
+      <c r="D33" s="31" t="n"/>
+      <c r="E33" s="31" t="n"/>
+      <c r="F33" s="32" t="n"/>
+      <c r="G33" s="31" t="n"/>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="33" t="n"/>
+      <c r="B34" s="33" t="n"/>
+      <c r="C34" s="33" t="n"/>
+      <c r="D34" s="33" t="n"/>
+      <c r="E34" s="33" t="n"/>
+      <c r="F34" s="34" t="n"/>
+      <c r="G34" s="33" t="n"/>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="31" t="n"/>
+      <c r="B35" s="31" t="n"/>
+      <c r="C35" s="31" t="n"/>
+      <c r="D35" s="31" t="n"/>
+      <c r="E35" s="31" t="n"/>
+      <c r="F35" s="32" t="n"/>
+      <c r="G35" s="31" t="n"/>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="33" t="n"/>
+      <c r="B36" s="33" t="n"/>
+      <c r="C36" s="33" t="n"/>
+      <c r="D36" s="33" t="n"/>
+      <c r="E36" s="33" t="n"/>
+      <c r="F36" s="34" t="n"/>
+      <c r="G36" s="33" t="n"/>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="31" t="n"/>
+      <c r="B37" s="31" t="n"/>
+      <c r="C37" s="31" t="n"/>
+      <c r="D37" s="31" t="n"/>
+      <c r="E37" s="31" t="n"/>
+      <c r="F37" s="32" t="n"/>
+      <c r="G37" s="31" t="n"/>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="33" t="n"/>
+      <c r="B38" s="33" t="n"/>
+      <c r="C38" s="33" t="n"/>
+      <c r="D38" s="33" t="n"/>
+      <c r="E38" s="33" t="n"/>
+      <c r="F38" s="34" t="n"/>
+      <c r="G38" s="33" t="n"/>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="31" t="n"/>
+      <c r="B39" s="31" t="n"/>
+      <c r="C39" s="31" t="n"/>
+      <c r="D39" s="31" t="n"/>
+      <c r="E39" s="31" t="n"/>
+      <c r="F39" s="32" t="n"/>
+      <c r="G39" s="31" t="n"/>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="33" t="n"/>
+      <c r="B40" s="33" t="n"/>
+      <c r="C40" s="33" t="n"/>
+      <c r="D40" s="33" t="n"/>
+      <c r="E40" s="33" t="n"/>
+      <c r="F40" s="34" t="n"/>
+      <c r="G40" s="33" t="n"/>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="31" t="n"/>
+      <c r="B41" s="31" t="n"/>
+      <c r="C41" s="31" t="n"/>
+      <c r="D41" s="31" t="n"/>
+      <c r="E41" s="31" t="n"/>
+      <c r="F41" s="32" t="n"/>
+      <c r="G41" s="31" t="n"/>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="33" t="n"/>
+      <c r="B42" s="33" t="n"/>
+      <c r="C42" s="33" t="n"/>
+      <c r="D42" s="33" t="n"/>
+      <c r="E42" s="33" t="n"/>
+      <c r="F42" s="34" t="n"/>
+      <c r="G42" s="33" t="n"/>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="31" t="n"/>
+      <c r="B43" s="31" t="n"/>
+      <c r="C43" s="31" t="n"/>
+      <c r="D43" s="31" t="n"/>
+      <c r="E43" s="31" t="n"/>
+      <c r="F43" s="32" t="n"/>
+      <c r="G43" s="31" t="n"/>
+    </row>
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="33" t="n"/>
+      <c r="B44" s="33" t="n"/>
+      <c r="C44" s="33" t="n"/>
+      <c r="D44" s="33" t="n"/>
+      <c r="E44" s="33" t="n"/>
+      <c r="F44" s="34" t="n"/>
+      <c r="G44" s="33" t="n"/>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="31" t="n"/>
+      <c r="B45" s="31" t="n"/>
+      <c r="C45" s="31" t="n"/>
+      <c r="D45" s="31" t="n"/>
+      <c r="E45" s="31" t="n"/>
+      <c r="F45" s="32" t="n"/>
+      <c r="G45" s="31" t="n"/>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="33" t="n"/>
+      <c r="B46" s="33" t="n"/>
+      <c r="C46" s="33" t="n"/>
+      <c r="D46" s="33" t="n"/>
+      <c r="E46" s="33" t="n"/>
+      <c r="F46" s="34" t="n"/>
+      <c r="G46" s="33" t="n"/>
+    </row>
+    <row r="47" ht="16" customHeight="1">
+      <c r="A47" s="31" t="n"/>
+      <c r="B47" s="31" t="n"/>
+      <c r="C47" s="31" t="n"/>
+      <c r="D47" s="31" t="n"/>
+      <c r="E47" s="31" t="n"/>
+      <c r="F47" s="32" t="n"/>
+      <c r="G47" s="31" t="n"/>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="A48" s="33" t="n"/>
+      <c r="B48" s="33" t="n"/>
+      <c r="C48" s="33" t="n"/>
+      <c r="D48" s="33" t="n"/>
+      <c r="E48" s="33" t="n"/>
+      <c r="F48" s="34" t="n"/>
+      <c r="G48" s="33" t="n"/>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="31" t="n"/>
+      <c r="B49" s="31" t="n"/>
+      <c r="C49" s="31" t="n"/>
+      <c r="D49" s="31" t="n"/>
+      <c r="E49" s="31" t="n"/>
+      <c r="F49" s="32" t="n"/>
+      <c r="G49" s="31" t="n"/>
+    </row>
+    <row r="50" ht="16" customHeight="1">
+      <c r="A50" s="33" t="n"/>
+      <c r="B50" s="33" t="n"/>
+      <c r="C50" s="33" t="n"/>
+      <c r="D50" s="33" t="n"/>
+      <c r="E50" s="33" t="n"/>
+      <c r="F50" s="34" t="n"/>
+      <c r="G50" s="33" t="n"/>
+    </row>
+    <row r="51" ht="16" customHeight="1">
+      <c r="A51" s="31" t="n"/>
+      <c r="B51" s="31" t="n"/>
+      <c r="C51" s="31" t="n"/>
+      <c r="D51" s="31" t="n"/>
+      <c r="E51" s="31" t="n"/>
+      <c r="F51" s="32" t="n"/>
+      <c r="G51" s="31" t="n"/>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="33" t="n"/>
+      <c r="B52" s="33" t="n"/>
+      <c r="C52" s="33" t="n"/>
+      <c r="D52" s="33" t="n"/>
+      <c r="E52" s="33" t="n"/>
+      <c r="F52" s="34" t="n"/>
+      <c r="G52" s="33" t="n"/>
+    </row>
+    <row r="53" ht="16" customHeight="1">
+      <c r="A53" s="31" t="n"/>
+      <c r="B53" s="31" t="n"/>
+      <c r="C53" s="31" t="n"/>
+      <c r="D53" s="31" t="n"/>
+      <c r="E53" s="31" t="n"/>
+      <c r="F53" s="32" t="n"/>
+      <c r="G53" s="31" t="n"/>
+    </row>
+    <row r="54" ht="16" customHeight="1">
+      <c r="A54" s="33" t="n"/>
+      <c r="B54" s="33" t="n"/>
+      <c r="C54" s="33" t="n"/>
+      <c r="D54" s="33" t="n"/>
+      <c r="E54" s="33" t="n"/>
+      <c r="F54" s="34" t="n"/>
+      <c r="G54" s="33" t="n"/>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="31" t="n"/>
+      <c r="B55" s="31" t="n"/>
+      <c r="C55" s="31" t="n"/>
+      <c r="D55" s="31" t="n"/>
+      <c r="E55" s="31" t="n"/>
+      <c r="F55" s="32" t="n"/>
+      <c r="G55" s="31" t="n"/>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="33" t="n"/>
+      <c r="B56" s="33" t="n"/>
+      <c r="C56" s="33" t="n"/>
+      <c r="D56" s="33" t="n"/>
+      <c r="E56" s="33" t="n"/>
+      <c r="F56" s="34" t="n"/>
+      <c r="G56" s="33" t="n"/>
+    </row>
+    <row r="57" ht="16" customHeight="1">
+      <c r="A57" s="31" t="n"/>
+      <c r="B57" s="31" t="n"/>
+      <c r="C57" s="31" t="n"/>
+      <c r="D57" s="31" t="n"/>
+      <c r="E57" s="31" t="n"/>
+      <c r="F57" s="32" t="n"/>
+      <c r="G57" s="31" t="n"/>
+    </row>
+    <row r="58" ht="16" customHeight="1">
+      <c r="A58" s="33" t="n"/>
+      <c r="B58" s="33" t="n"/>
+      <c r="C58" s="33" t="n"/>
+      <c r="D58" s="33" t="n"/>
+      <c r="E58" s="33" t="n"/>
+      <c r="F58" s="34" t="n"/>
+      <c r="G58" s="33" t="n"/>
+    </row>
+    <row r="59" ht="16" customHeight="1">
+      <c r="A59" s="31" t="n"/>
+      <c r="B59" s="31" t="n"/>
+      <c r="C59" s="31" t="n"/>
+      <c r="D59" s="31" t="n"/>
+      <c r="E59" s="31" t="n"/>
+      <c r="F59" s="32" t="n"/>
+      <c r="G59" s="31" t="n"/>
+    </row>
+    <row r="60" ht="16" customHeight="1">
+      <c r="A60" s="33" t="n"/>
+      <c r="B60" s="33" t="n"/>
+      <c r="C60" s="33" t="n"/>
+      <c r="D60" s="33" t="n"/>
+      <c r="E60" s="33" t="n"/>
+      <c r="F60" s="34" t="n"/>
+      <c r="G60" s="33" t="n"/>
+    </row>
+    <row r="61" ht="16" customHeight="1">
+      <c r="A61" s="31" t="n"/>
+      <c r="B61" s="31" t="n"/>
+      <c r="C61" s="31" t="n"/>
+      <c r="D61" s="31" t="n"/>
+      <c r="E61" s="31" t="n"/>
+      <c r="F61" s="32" t="n"/>
+      <c r="G61" s="31" t="n"/>
+    </row>
+    <row r="62" ht="16" customHeight="1">
+      <c r="A62" s="33" t="n"/>
+      <c r="B62" s="33" t="n"/>
+      <c r="C62" s="33" t="n"/>
+      <c r="D62" s="33" t="n"/>
+      <c r="E62" s="33" t="n"/>
+      <c r="F62" s="34" t="n"/>
+      <c r="G62" s="33" t="n"/>
+    </row>
+    <row r="63" ht="16" customHeight="1">
+      <c r="A63" s="31" t="n"/>
+      <c r="B63" s="31" t="n"/>
+      <c r="C63" s="31" t="n"/>
+      <c r="D63" s="31" t="n"/>
+      <c r="E63" s="31" t="n"/>
+      <c r="F63" s="32" t="n"/>
+      <c r="G63" s="31" t="n"/>
+    </row>
+    <row r="64" ht="16" customHeight="1">
+      <c r="A64" s="33" t="n"/>
+      <c r="B64" s="33" t="n"/>
+      <c r="C64" s="33" t="n"/>
+      <c r="D64" s="33" t="n"/>
+      <c r="E64" s="33" t="n"/>
+      <c r="F64" s="34" t="n"/>
+      <c r="G64" s="33" t="n"/>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>RESUMEN AUTOMATICO (se calcula solo a medida que cargas filas arriba)</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="n"/>
+      <c r="C66" s="5" t="n"/>
+      <c r="D66" s="5" t="n"/>
+      <c r="E66" s="5" t="n"/>
+      <c r="F66" s="5" t="n"/>
+      <c r="G66" s="5" t="n"/>
+    </row>
+    <row r="67" ht="16" customHeight="1">
+      <c r="A67" s="35" t="inlineStr">
+        <is>
+          <t>Total Nucleo 1</t>
+        </is>
+      </c>
+      <c r="B67" s="20">
+        <f>SUMIF($D$5:$D$64,"Nucleo 1",$F$5:$F$64)</f>
+        <v/>
+      </c>
+      <c r="C67" s="36" t="n"/>
+      <c r="D67" s="36" t="n"/>
+      <c r="E67" s="36" t="n"/>
+      <c r="F67" s="36" t="n"/>
+      <c r="G67" s="36" t="n"/>
+    </row>
+    <row r="68" ht="16" customHeight="1">
+      <c r="A68" s="35" t="inlineStr">
+        <is>
+          <t>Total Nucleo 2</t>
+        </is>
+      </c>
+      <c r="B68" s="20">
+        <f>SUMIF($D$5:$D$64,"Nucleo 2",$F$5:$F$64)</f>
+        <v/>
+      </c>
+      <c r="C68" s="36" t="n"/>
+      <c r="D68" s="36" t="n"/>
+      <c r="E68" s="36" t="n"/>
+      <c r="F68" s="36" t="n"/>
+      <c r="G68" s="36" t="n"/>
+    </row>
+    <row r="69" ht="16" customHeight="1">
+      <c r="A69" s="35" t="inlineStr">
+        <is>
+          <t>Total Nucleo 3</t>
+        </is>
+      </c>
+      <c r="B69" s="20">
+        <f>SUMIF($D$5:$D$64,"Nucleo 3",$F$5:$F$64)</f>
+        <v/>
+      </c>
+      <c r="C69" s="36" t="n"/>
+      <c r="D69" s="36" t="n"/>
+      <c r="E69" s="36" t="n"/>
+      <c r="F69" s="36" t="n"/>
+      <c r="G69" s="36" t="n"/>
+    </row>
+    <row r="70" ht="16" customHeight="1">
+      <c r="A70" s="35" t="inlineStr">
+        <is>
+          <t>Total Compartido/Todos</t>
+        </is>
+      </c>
+      <c r="B70" s="20">
+        <f>SUMIF($D$5:$D$64,"Compartido/Todos",$F$5:$F$64)</f>
+        <v/>
+      </c>
+      <c r="C70" s="36" t="n"/>
+      <c r="D70" s="36" t="n"/>
+      <c r="E70" s="36" t="n"/>
+      <c r="F70" s="36" t="n"/>
+      <c r="G70" s="36" t="n"/>
+    </row>
+    <row r="71" ht="16" customHeight="1">
+      <c r="A71" s="35" t="inlineStr">
+        <is>
+          <t>Costo Nico (50% Nucleo 3)</t>
+        </is>
+      </c>
+      <c r="B71" s="20">
+        <f>B69/2</f>
+        <v/>
+      </c>
+      <c r="C71" s="36" t="n"/>
+      <c r="D71" s="36" t="n"/>
+      <c r="E71" s="36" t="n"/>
+      <c r="F71" s="36" t="n"/>
+      <c r="G71" s="36" t="n"/>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="24" t="inlineStr">
+        <is>
+          <t>TOTAL REGISTRADO</t>
+        </is>
+      </c>
+      <c r="B72" s="26">
+        <f>SUM($F$5:$F$64)</f>
+        <v/>
+      </c>
+      <c r="C72" s="25" t="n"/>
+      <c r="D72" s="25" t="n"/>
+      <c r="E72" s="25" t="n"/>
+      <c r="F72" s="25" t="n"/>
+      <c r="G72" s="25" t="n"/>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>DEUDAS ENTRE PERSONAS (adelantos de un integrante a nombre de otros)</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="n"/>
+      <c r="C75" s="5" t="n"/>
+      <c r="D75" s="5" t="n"/>
+      <c r="E75" s="5" t="n"/>
+      <c r="F75" s="5" t="n"/>
+      <c r="G75" s="5" t="n"/>
+    </row>
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="29" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B76" s="29" t="inlineStr">
+        <is>
+          <t>Adelanto pagado por</t>
+        </is>
+      </c>
+      <c r="C76" s="29" t="inlineStr">
+        <is>
+          <t>A cargo de</t>
+        </is>
+      </c>
+      <c r="D76" s="29" t="inlineStr">
+        <is>
+          <t>Monto USD</t>
+        </is>
+      </c>
+      <c r="E76" s="29" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="F76" s="37" t="n"/>
+      <c r="G76" s="38" t="n"/>
+    </row>
+    <row r="77" ht="40" customHeight="1">
+      <c r="A77" s="19" t="inlineStr">
+        <is>
+          <t>Universal Dockside (reserva conjunta 63W124U2: Florencia, German, Natalia, Nicolas)</t>
+        </is>
+      </c>
+      <c r="B77" s="19" t="inlineStr">
+        <is>
+          <t>German Agullo (pago la reserva completa)</t>
+        </is>
+      </c>
+      <c r="C77" s="19" t="inlineStr">
+        <is>
+          <t>Nicolas y Natalia (Nucleo 3) le deben a German la mitad de esta reserva + lo que falte pagar</t>
+        </is>
+      </c>
+      <c r="D77" s="20">
+        <f>'Matriz Financiera'!F6</f>
+        <v/>
+      </c>
+      <c r="E77" s="39" t="inlineStr">
+        <is>
+          <t>Pendiente de liquidar con German</t>
+        </is>
+      </c>
+      <c r="F77" s="36" t="n"/>
+      <c r="G77" s="36" t="n"/>
+    </row>
+    <row r="78" ht="40" customHeight="1">
+      <c r="A78" s="19" t="inlineStr">
+        <is>
+          <t>Disney Art of Animation (reserva #43028783: Natalia, Nicolas)</t>
+        </is>
+      </c>
+      <c r="B78" s="19" t="inlineStr">
+        <is>
+          <t>Nicolas y Natalia (pagan directo, sin intermediario)</t>
+        </is>
+      </c>
+      <c r="C78" s="19" t="inlineStr">
+        <is>
+          <t>N/A - no genera deuda entre personas</t>
+        </is>
+      </c>
+      <c r="D78" s="20">
+        <f>'Matriz Financiera'!F5</f>
+        <v/>
+      </c>
+      <c r="E78" s="39" t="inlineStr">
+        <is>
+          <t>Gestionado directamente por Nucleo 3</t>
+        </is>
+      </c>
+      <c r="F78" s="36" t="n"/>
+      <c r="G78" s="36" t="n"/>
+    </row>
+    <row r="80" ht="30" customHeight="1">
+      <c r="A80" s="40" t="inlineStr">
+        <is>
+          <t>El monto de la fila Universal esta enlazado por formula a la Matriz Financiera (Nucleo 3 = mitad de la reserva conjunta 63W124U2). Incluye la sena ya pagada y el saldo que falte liquidar con German a medida que se vaya pagando la reserva completa.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="E77:G77"/>
+    <mergeCell ref="A66:G66"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A80:G80"/>
+    <mergeCell ref="E78:G78"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="E76:G76"/>
+    <mergeCell ref="A75:G75"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="B5:B64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Vuelos,Disney,Universal,Hospedaje Miami,Auto/Transporte,Comida,Compras,Seguro,Propinas,Otro"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D5:D64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Nucleo 1,Nucleo 2,Nucleo 3,Compartido/Todos"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ITINERARIO FLASH - CALENDARIO FEBRERO 2027</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="29" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B3" s="28" t="inlineStr">
+      <c r="B3" s="29" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="C3" s="29" t="inlineStr">
         <is>
           <t>Momento del dia</t>
         </is>
       </c>
-      <c r="C3" s="28" t="inlineStr">
+      <c r="D3" s="29" t="inlineStr">
         <is>
           <t>Actividad / Lugar</t>
         </is>
       </c>
-      <c r="D3" s="28" t="inlineStr">
+      <c r="E3" s="29" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="F3" s="29" t="inlineStr">
         <is>
           <t>Tip pragmatico</t>
         </is>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>05-feb (vie)</t>
         </is>
       </c>
-      <c r="B4" s="30" t="inlineStr">
-        <is>
-          <t>Madrugada/Manana</t>
-        </is>
-      </c>
-      <c r="C4" s="30" t="inlineStr">
+      <c r="B4" s="41" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="inlineStr">
+        <is>
+          <t>Manana</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>Vuelo AA982 EZE -&gt; MIA (10:10 a 17:20)</t>
         </is>
       </c>
-      <c r="D4" s="30" t="inlineStr">
+      <c r="E4" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
         <is>
           <t>-&gt; Check-in online 24h antes; llegar a EZE con 3h de anticipacion por ser vuelo internacional B1/B2.</t>
         </is>
@@ -1496,39 +2431,59 @@
           <t>05-feb (vie)</t>
         </is>
       </c>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B5" s="41" t="inlineStr">
+        <is>
+          <t>18:56</t>
+        </is>
+      </c>
+      <c r="C5" s="41" t="inlineStr">
         <is>
           <t>Tarde/Noche</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>Conexion AA1856 MIA -&gt; MCO (18:56 a 20:15)</t>
         </is>
       </c>
-      <c r="D5" s="19" t="inlineStr">
+      <c r="E5" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
         <is>
           <t>-&gt; Conexion corta (1h36) dentro del mismo aeropuerto MIA; no hace falta retirar equipaje si esta chequeado hasta MCO.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>05-feb (vie)</t>
         </is>
       </c>
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
         <is>
           <t>Noche</t>
         </is>
       </c>
-      <c r="C6" s="30" t="inlineStr">
+      <c r="D6" s="19" t="inlineStr">
         <is>
           <t>Llegada a Orlando -&gt; Check-in Disney's Art of Animation</t>
         </is>
       </c>
-      <c r="D6" s="30" t="inlineStr">
+      <c r="E6" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
         <is>
           <t>-&gt; Traslado en 2 UberXL (7 pax + 21 bultos); pedir con anticipacion por horario nocturno.</t>
         </is>
@@ -1540,39 +2495,59 @@
           <t>06-feb (sab)</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>Parque Disney 1</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="E7" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>-&gt; Comprar Lightning Lane Multi Pass apenas abre la app a las 7am.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>07-feb (dom)</t>
         </is>
       </c>
-      <c r="B8" s="30" t="inlineStr">
+      <c r="B8" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C8" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C8" s="30" t="inlineStr">
+      <c r="D8" s="19" t="inlineStr">
         <is>
           <t>Parque Disney 2</t>
         </is>
       </c>
-      <c r="D8" s="30" t="inlineStr">
+      <c r="E8" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
         <is>
           <t>-&gt; Reservar restaurante con Advance Dining Reservation si se sale del Quick-Service.</t>
         </is>
@@ -1584,39 +2559,59 @@
           <t>08-feb (lun)</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B9" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C9" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>Parque Disney 3</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
+      <c r="E9" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
         <is>
           <t>-&gt; Dia de mayor concurrencia -&gt; priorizar atracciones top apenas abre el parque.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>09-feb (mar)</t>
         </is>
       </c>
-      <c r="B10" s="30" t="inlineStr">
+      <c r="B10" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C10" s="30" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>Parque Disney 4</t>
         </is>
       </c>
-      <c r="D10" s="30" t="inlineStr">
+      <c r="E10" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
         <is>
           <t>-&gt; Aprovechar Extra Magic Hours si el hotel las tiene habilitadas ese dia.</t>
         </is>
@@ -1628,39 +2623,59 @@
           <t>10-feb (mie)</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B11" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C11" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>Parque Disney 5</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="E11" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
         <is>
           <t>-&gt; Guardar el ultimo dia de ticket Disney para el parque favorito del grupo.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>11-feb (jue)</t>
         </is>
       </c>
-      <c r="B12" s="30" t="inlineStr">
+      <c r="B12" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C12" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C12" s="30" t="inlineStr">
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>Descanso / Compras en Orlando International Premium Outlets</t>
         </is>
       </c>
-      <c r="D12" s="30" t="inlineStr">
+      <c r="E12" s="43" t="inlineStr">
+        <is>
+          <t>Por organizar</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
         <is>
           <t>-&gt; Uber compartido con otras familias del resort para bajar el costo del traslado.</t>
         </is>
@@ -1672,39 +2687,59 @@
           <t>12-feb (vie)</t>
         </is>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
         <is>
           <t>Manana</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>Check-out Disney -&gt; Check-in Universal Dockside Inn</t>
         </is>
       </c>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="E13" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
         <is>
           <t>-&gt; Guardar equipaje en Bell Services de Disney si el check-in de Universal es mas tarde.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="29" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>12-feb (vie)</t>
         </is>
       </c>
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B14" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C14" s="41" t="inlineStr">
         <is>
           <t>Tarde</t>
         </is>
       </c>
-      <c r="C14" s="30" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>Early Park Admission Universal (segun ticket)</t>
         </is>
       </c>
-      <c r="D14" s="30" t="inlineStr">
+      <c r="E14" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
         <is>
           <t>-&gt; Usar el transporte gratuito del hotel Dockside en vez de Uber.</t>
         </is>
@@ -1716,39 +2751,59 @@
           <t>13-feb (sab)</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B15" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C15" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>Universal Epic Universe</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="E15" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
         <is>
           <t>-&gt; Llegar 45 min antes de la apertura general por controles de seguridad reforzados.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="34" customHeight="1">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>14-feb (dom)</t>
         </is>
       </c>
-      <c r="B16" s="30" t="inlineStr">
+      <c r="B16" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C16" s="30" t="inlineStr">
+      <c r="D16" s="19" t="inlineStr">
         <is>
           <t>Universal's Islands of Adventure</t>
         </is>
       </c>
-      <c r="D16" s="30" t="inlineStr">
+      <c r="E16" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
         <is>
           <t>-&gt; Ir directo a VelociCoaster apenas abre el parque.</t>
         </is>
@@ -1760,39 +2815,59 @@
           <t>15-feb (lun)</t>
         </is>
       </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B17" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C17" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>Dia libre / Compras</t>
         </is>
       </c>
-      <c r="D17" s="19" t="inlineStr">
+      <c r="E17" s="43" t="inlineStr">
+        <is>
+          <t>Por organizar</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
         <is>
           <t>-&gt; Aprovechar para lavar ropa; la mayoria de los Dockside tienen lavanderia self-service.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="34" customHeight="1">
-      <c r="A18" s="29" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>16-feb (mar)</t>
         </is>
       </c>
-      <c r="B18" s="30" t="inlineStr">
+      <c r="B18" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C18" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C18" s="30" t="inlineStr">
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>Universal Studios Florida</t>
         </is>
       </c>
-      <c r="D18" s="30" t="inlineStr">
+      <c r="E18" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
         <is>
           <t>-&gt; Usar el Hogwarts Express (Park-to-Park) para moverse entre parques sin volver a la entrada.</t>
         </is>
@@ -1804,39 +2879,59 @@
           <t>17-feb (mie)</t>
         </is>
       </c>
-      <c r="B19" s="19" t="inlineStr">
+      <c r="B19" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C19" s="41" t="inlineStr">
         <is>
           <t>Manana</t>
         </is>
       </c>
-      <c r="C19" s="19" t="inlineStr">
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>Check-out Universal -&gt; 2 UberXL a MCO</t>
         </is>
       </c>
-      <c r="D19" s="19" t="inlineStr">
+      <c r="E19" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
         <is>
           <t>-&gt; Salir con margen: 21 bultos de equipaje hacen mas lento el check-in en el aeropuerto domestico.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>17-feb (mie)</t>
         </is>
       </c>
-      <c r="B20" s="30" t="inlineStr">
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C20" s="41" t="inlineStr">
         <is>
           <t>Manana</t>
         </is>
       </c>
-      <c r="C20" s="30" t="inlineStr">
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>Vuelo AA1741 MCO -&gt; MIA (10:00 a 11:20)</t>
         </is>
       </c>
-      <c r="D20" s="30" t="inlineStr">
+      <c r="E20" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
         <is>
           <t>-&gt; Vuelo corto domestico; despachar valijas grandes igual (no entran como carry-on).</t>
         </is>
@@ -1848,39 +2943,59 @@
           <t>17-feb (mie)</t>
         </is>
       </c>
-      <c r="B21" s="19" t="inlineStr">
+      <c r="B21" s="41" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="C21" s="41" t="inlineStr">
         <is>
           <t>Mediodia/Tarde</t>
         </is>
       </c>
-      <c r="C21" s="19" t="inlineStr">
+      <c r="D21" s="19" t="inlineStr">
         <is>
           <t>Llegada Miami -&gt; Check-in departamento Hollywood Beach + retiro de minivan</t>
         </is>
       </c>
-      <c r="D21" s="19" t="inlineStr">
+      <c r="E21" s="43" t="inlineStr">
+        <is>
+          <t>Por organizar</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
         <is>
           <t>-&gt; Retirar la minivan (Chrysler Pacifica/Kia Carnival) directo en el aeropuerto MIA para evitar un traslado extra.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="29" t="inlineStr">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>18-feb (jue)</t>
         </is>
       </c>
-      <c r="B22" s="30" t="inlineStr">
+      <c r="B22" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C22" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C22" s="30" t="inlineStr">
+      <c r="D22" s="19" t="inlineStr">
         <is>
           <t>Hollywood Beach - playa y Broadwalk</t>
         </is>
       </c>
-      <c r="D22" s="30" t="inlineStr">
+      <c r="E22" s="43" t="inlineStr">
+        <is>
+          <t>Por organizar</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
         <is>
           <t>-&gt; Comprar en Publix o Walmart apenas se llega para no depender de delivery los primeros dias.</t>
         </is>
@@ -1892,39 +3007,59 @@
           <t>19-feb (vie)</t>
         </is>
       </c>
-      <c r="B23" s="19" t="inlineStr">
+      <c r="B23" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C23" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C23" s="19" t="inlineStr">
+      <c r="D23" s="19" t="inlineStr">
         <is>
           <t>Dia libre Miami / Excursion opcional</t>
         </is>
       </c>
-      <c r="D23" s="19" t="inlineStr">
+      <c r="E23" s="43" t="inlineStr">
+        <is>
+          <t>Por organizar</t>
+        </is>
+      </c>
+      <c r="F23" s="19" t="inlineStr">
         <is>
           <t>-&gt; Cargar SunPass antes de salir a la ruta para evitar recargos por peaje sin transponder.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="34" customHeight="1">
-      <c r="A24" s="29" t="inlineStr">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>20-feb (sab)</t>
         </is>
       </c>
-      <c r="B24" s="30" t="inlineStr">
+      <c r="B24" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C24" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C24" s="30" t="inlineStr">
+      <c r="D24" s="19" t="inlineStr">
         <is>
           <t>Miami - paseo urbano (Wynwood / South Beach)</t>
         </is>
       </c>
-      <c r="D24" s="30" t="inlineStr">
+      <c r="E24" s="43" t="inlineStr">
+        <is>
+          <t>Por organizar</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
         <is>
           <t>-&gt; Estacionamiento pago en South Beach; verificar tarifa horaria antes de dejar la minivan.</t>
         </is>
@@ -1936,39 +3071,59 @@
           <t>21-feb (dom)</t>
         </is>
       </c>
-      <c r="B25" s="19" t="inlineStr">
+      <c r="B25" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C25" s="41" t="inlineStr">
         <is>
           <t>Todo el dia</t>
         </is>
       </c>
-      <c r="C25" s="19" t="inlineStr">
+      <c r="D25" s="19" t="inlineStr">
         <is>
           <t>Ultimo dia libre + preparar valijas</t>
         </is>
       </c>
-      <c r="D25" s="19" t="inlineStr">
+      <c r="E25" s="43" t="inlineStr">
+        <is>
+          <t>Por organizar</t>
+        </is>
+      </c>
+      <c r="F25" s="19" t="inlineStr">
         <is>
           <t>-&gt; Revisar franquicia de equipaje del vuelo internacional (distinta a la domestica) antes de repartir compras.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="29" t="inlineStr">
+      <c r="A26" s="18" t="inlineStr">
         <is>
           <t>22-feb (lun)</t>
         </is>
       </c>
-      <c r="B26" s="30" t="inlineStr">
+      <c r="B26" s="41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C26" s="41" t="inlineStr">
         <is>
           <t>Tarde</t>
         </is>
       </c>
-      <c r="C26" s="30" t="inlineStr">
+      <c r="D26" s="19" t="inlineStr">
         <is>
           <t>Check-out departamento + devolucion minivan en MIA</t>
         </is>
       </c>
-      <c r="D26" s="30" t="inlineStr">
+      <c r="E26" s="43" t="inlineStr">
+        <is>
+          <t>Por organizar</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
         <is>
           <t>-&gt; Devolver el tanque lleno para evitar el cargo de combustible de la rentadora.</t>
         </is>
@@ -1980,31 +3135,49 @@
           <t>22-feb (lun)</t>
         </is>
       </c>
-      <c r="B27" s="19" t="inlineStr">
+      <c r="B27" s="41" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C27" s="41" t="inlineStr">
         <is>
           <t>Noche</t>
         </is>
       </c>
-      <c r="C27" s="19" t="inlineStr">
+      <c r="D27" s="19" t="inlineStr">
         <is>
           <t>Vuelo AA931 MIA -&gt; EZE (20:15, llega 07:25 del 23-feb)</t>
         </is>
       </c>
-      <c r="D27" s="19" t="inlineStr">
+      <c r="E27" s="42" t="inlineStr">
+        <is>
+          <t>Confirmado</t>
+        </is>
+      </c>
+      <c r="F27" s="19" t="inlineStr">
         <is>
           <t>-&gt; Llegar a MIA con 3.5h de anticipacion por ser vuelo internacional con 7 pasajeros y equipaje voluminoso.</t>
         </is>
       </c>
     </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="44" t="inlineStr">
+        <is>
+          <t>Confirmado = ya reservado/facturado (vuelos, Disney, Universal). Por organizar = todavia sin reserva (Hollywood Beach, minivan, dias libres de Miami).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A29:F29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2052,217 +3225,217 @@
       <c r="H3" s="5" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>Vuelo</t>
         </is>
       </c>
-      <c r="C4" s="28" t="inlineStr">
+      <c r="C4" s="29" t="inlineStr">
         <is>
           <t>Tramo</t>
         </is>
       </c>
-      <c r="D4" s="28" t="inlineStr">
+      <c r="D4" s="29" t="inlineStr">
         <is>
           <t>Salida</t>
         </is>
       </c>
-      <c r="E4" s="28" t="inlineStr">
+      <c r="E4" s="29" t="inlineStr">
         <is>
           <t>Llegada</t>
         </is>
       </c>
-      <c r="F4" s="28" t="inlineStr">
+      <c r="F4" s="29" t="inlineStr">
         <is>
           <t>Duracion</t>
         </is>
       </c>
-      <c r="G4" s="28" t="inlineStr">
+      <c r="G4" s="29" t="inlineStr">
         <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="H4" s="28" t="inlineStr">
+      <c r="H4" s="29" t="inlineStr">
         <is>
           <t>Equipo</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="31" t="inlineStr">
+      <c r="A5" s="41" t="inlineStr">
         <is>
           <t>05-feb-2027</t>
         </is>
       </c>
-      <c r="B5" s="31" t="inlineStr">
+      <c r="B5" s="41" t="inlineStr">
         <is>
           <t>AA 982</t>
         </is>
       </c>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="41" t="inlineStr">
         <is>
           <t>EZE -&gt; MIA</t>
         </is>
       </c>
-      <c r="D5" s="31" t="inlineStr">
+      <c r="D5" s="41" t="inlineStr">
         <is>
           <t>10:10</t>
         </is>
       </c>
-      <c r="E5" s="31" t="inlineStr">
+      <c r="E5" s="41" t="inlineStr">
         <is>
           <t>17:20</t>
         </is>
       </c>
-      <c r="F5" s="31" t="inlineStr">
+      <c r="F5" s="41" t="inlineStr">
         <is>
           <t>9:10</t>
         </is>
       </c>
-      <c r="G5" s="31" t="inlineStr">
+      <c r="G5" s="41" t="inlineStr">
         <is>
           <t>P (EZE, salida)</t>
         </is>
       </c>
-      <c r="H5" s="31" t="inlineStr">
+      <c r="H5" s="41" t="inlineStr">
         <is>
           <t>Boeing 787-8</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="A6" s="41" t="inlineStr">
         <is>
           <t>05-feb-2027</t>
         </is>
       </c>
-      <c r="B6" s="31" t="inlineStr">
+      <c r="B6" s="41" t="inlineStr">
         <is>
           <t>AA 1856</t>
         </is>
       </c>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="C6" s="41" t="inlineStr">
         <is>
           <t>MIA -&gt; MCO</t>
         </is>
       </c>
-      <c r="D6" s="31" t="inlineStr">
+      <c r="D6" s="41" t="inlineStr">
         <is>
           <t>18:56</t>
         </is>
       </c>
-      <c r="E6" s="31" t="inlineStr">
+      <c r="E6" s="41" t="inlineStr">
         <is>
           <t>20:15</t>
         </is>
       </c>
-      <c r="F6" s="31" t="inlineStr">
+      <c r="F6" s="41" t="inlineStr">
         <is>
           <t>1:19</t>
         </is>
       </c>
-      <c r="G6" s="31" t="inlineStr">
+      <c r="G6" s="41" t="inlineStr">
         <is>
           <t>B (MCO, llegada)</t>
         </is>
       </c>
-      <c r="H6" s="31" t="inlineStr">
+      <c r="H6" s="41" t="inlineStr">
         <is>
           <t>Boeing 737 MAX 8</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="31" t="inlineStr">
+      <c r="A7" s="41" t="inlineStr">
         <is>
           <t>17-feb-2027</t>
         </is>
       </c>
-      <c r="B7" s="31" t="inlineStr">
+      <c r="B7" s="41" t="inlineStr">
         <is>
           <t>AA 1741</t>
         </is>
       </c>
-      <c r="C7" s="31" t="inlineStr">
+      <c r="C7" s="41" t="inlineStr">
         <is>
           <t>MCO -&gt; MIA</t>
         </is>
       </c>
-      <c r="D7" s="31" t="inlineStr">
+      <c r="D7" s="41" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="E7" s="31" t="inlineStr">
+      <c r="E7" s="41" t="inlineStr">
         <is>
           <t>11:20</t>
         </is>
       </c>
-      <c r="F7" s="31" t="inlineStr">
+      <c r="F7" s="41" t="inlineStr">
         <is>
           <t>1:20</t>
         </is>
       </c>
-      <c r="G7" s="31" t="inlineStr">
+      <c r="G7" s="41" t="inlineStr">
         <is>
           <t>B (MCO, salida)</t>
         </is>
       </c>
-      <c r="H7" s="31" t="inlineStr">
+      <c r="H7" s="41" t="inlineStr">
         <is>
           <t>Boeing 737 MAX 8</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="31" t="inlineStr">
+      <c r="A8" s="41" t="inlineStr">
         <is>
           <t>22-feb-2027</t>
         </is>
       </c>
-      <c r="B8" s="31" t="inlineStr">
+      <c r="B8" s="41" t="inlineStr">
         <is>
           <t>AA 931</t>
         </is>
       </c>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="C8" s="41" t="inlineStr">
         <is>
           <t>MIA -&gt; EZE</t>
         </is>
       </c>
-      <c r="D8" s="31" t="inlineStr">
+      <c r="D8" s="41" t="inlineStr">
         <is>
           <t>20:15</t>
         </is>
       </c>
-      <c r="E8" s="31" t="inlineStr">
+      <c r="E8" s="41" t="inlineStr">
         <is>
           <t>07:25 (23-feb)</t>
         </is>
       </c>
-      <c r="F8" s="31" t="inlineStr">
+      <c r="F8" s="41" t="inlineStr">
         <is>
           <t>9:10</t>
         </is>
       </c>
-      <c r="G8" s="31" t="inlineStr">
+      <c r="G8" s="41" t="inlineStr">
         <is>
           <t>IA (EZE, llegada)</t>
         </is>
       </c>
-      <c r="H8" s="31" t="inlineStr">
+      <c r="H8" s="41" t="inlineStr">
         <is>
           <t>Boeing 777-200/200ER</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="44" t="inlineStr">
         <is>
           <t>Nota: costo de los pasajes no disponible en el e-ticket. Ver fila 'Vuelos' en Matriz Financiera (celda A COMPLETAR).</t>
         </is>
@@ -2283,23 +3456,23 @@
       <c r="H12" s="5" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="33" t="inlineStr">
+      <c r="A13" s="45" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B13" s="33" t="inlineStr">
+      <c r="B13" s="45" t="inlineStr">
         <is>
           <t>Detalle</t>
         </is>
       </c>
-      <c r="C13" s="34" t="n"/>
-      <c r="D13" s="34" t="n"/>
-      <c r="E13" s="34" t="n"/>
-      <c r="F13" s="35" t="n"/>
+      <c r="C13" s="37" t="n"/>
+      <c r="D13" s="37" t="n"/>
+      <c r="E13" s="37" t="n"/>
+      <c r="F13" s="38" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="36" t="inlineStr">
+      <c r="A14" s="33" t="inlineStr">
         <is>
           <t>Tarifa base</t>
         </is>
@@ -2309,16 +3482,16 @@
           <t>Minivan 7 pax (Chrysler Pacifica / Kia Carnival), 5 dias, retiro/devolucion en MIA</t>
         </is>
       </c>
-      <c r="C14" s="37" t="n"/>
-      <c r="D14" s="37" t="n"/>
-      <c r="E14" s="37" t="n"/>
-      <c r="F14" s="37" t="n"/>
+      <c r="C14" s="36" t="n"/>
+      <c r="D14" s="36" t="n"/>
+      <c r="E14" s="36" t="n"/>
+      <c r="F14" s="36" t="n"/>
       <c r="G14" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="36" t="inlineStr">
+      <c r="A15" s="33" t="inlineStr">
         <is>
           <t>Seguro CDW</t>
         </is>
@@ -2328,16 +3501,16 @@
           <t>Collision Damage Waiver. Verificar cobertura Visa Signature/AIG del titular antes de contratarlo con la rentadora.</t>
         </is>
       </c>
-      <c r="C15" s="37" t="n"/>
-      <c r="D15" s="37" t="n"/>
-      <c r="E15" s="37" t="n"/>
-      <c r="F15" s="37" t="n"/>
+      <c r="C15" s="36" t="n"/>
+      <c r="D15" s="36" t="n"/>
+      <c r="E15" s="36" t="n"/>
+      <c r="F15" s="36" t="n"/>
       <c r="G15" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="36" t="inlineStr">
+      <c r="A16" s="33" t="inlineStr">
         <is>
           <t>Seguro LIS</t>
         </is>
@@ -2347,16 +3520,16 @@
           <t>Liability Insurance Supplement</t>
         </is>
       </c>
-      <c r="C16" s="37" t="n"/>
-      <c r="D16" s="37" t="n"/>
-      <c r="E16" s="37" t="n"/>
-      <c r="F16" s="37" t="n"/>
+      <c r="C16" s="36" t="n"/>
+      <c r="D16" s="36" t="n"/>
+      <c r="E16" s="36" t="n"/>
+      <c r="F16" s="36" t="n"/>
       <c r="G16" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="36" t="inlineStr">
+      <c r="A17" s="33" t="inlineStr">
         <is>
           <t>Peajes / SunPass</t>
         </is>
@@ -2366,16 +3539,16 @@
           <t>Transponder o pase electronico para autopistas de Florida durante los 5 dias</t>
         </is>
       </c>
-      <c r="C17" s="37" t="n"/>
-      <c r="D17" s="37" t="n"/>
-      <c r="E17" s="37" t="n"/>
-      <c r="F17" s="37" t="n"/>
+      <c r="C17" s="36" t="n"/>
+      <c r="D17" s="36" t="n"/>
+      <c r="E17" s="36" t="n"/>
+      <c r="F17" s="36" t="n"/>
       <c r="G17" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="36" t="inlineStr">
+      <c r="A18" s="33" t="inlineStr">
         <is>
           <t>Estacionamiento Hollywood</t>
         </is>
@@ -2385,16 +3558,16 @@
           <t>Estacionamiento del departamento/edificio en Hollywood Beach</t>
         </is>
       </c>
-      <c r="C18" s="37" t="n"/>
-      <c r="D18" s="37" t="n"/>
-      <c r="E18" s="37" t="n"/>
-      <c r="F18" s="37" t="n"/>
+      <c r="C18" s="36" t="n"/>
+      <c r="D18" s="36" t="n"/>
+      <c r="E18" s="36" t="n"/>
+      <c r="F18" s="36" t="n"/>
       <c r="G18" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="38" t="inlineStr">
+      <c r="A19" s="46" t="inlineStr">
         <is>
           <t>SUBTOTAL ALQUILER AUTO</t>
         </is>
@@ -2404,7 +3577,7 @@
       <c r="D19" s="25" t="n"/>
       <c r="E19" s="25" t="n"/>
       <c r="F19" s="25" t="n"/>
-      <c r="G19" s="39">
+      <c r="G19" s="47">
         <f>SUM(G14:G18)</f>
         <v/>
       </c>
@@ -2435,7 +3608,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2504,7 +3677,7 @@
       </c>
     </row>
     <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="41" t="inlineStr">
+      <c r="A13" s="48" t="inlineStr">
         <is>
           <t>C_total_grupo = N x ( C_hospedaje + C_atracciones + n x (C_comida + C_transporte_local) + C_seguro )</t>
         </is>

</xml_diff>

<commit_message>
Gastos reales via chat en lugar de carga manual en Excel
El Registro de Gastos ahora lee de gastos_registrados.json en vez de
depender de que Nico tipee en la planilla. El flujo pasa a ser: Nico
cuenta el gasto por chat, se agrega una entrada al JSON y se regenera
el xlsx (mismo archivo/branch, siempre actualizado).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019LrLKneXbkjTi7bzStorH9
</commit_message>
<xml_diff>
--- a/Presupuesto_Florida_2027_Nico.xlsx
+++ b/Presupuesto_Florida_2027_Nico.xlsx
@@ -945,7 +945,7 @@
     <row r="21" ht="26" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>• Pestana 3 (Registro de Gastos): hoja de carga MANUAL para que Nico anote los gastos reales dia a dia (Uber, comidas, compras, etc.). Los totales por nucleo se calculan solos con formulas.</t>
+          <t>• Pestana 3 (Registro de Gastos): Nico le cuenta los gastos reales a Claude por chat y esta hoja se mantiene actualizada sola. Los totales por nucleo se calculan solos con formulas.</t>
         </is>
       </c>
     </row>
@@ -1468,7 +1468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1483,7 +1483,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>REGISTRO DE GASTOS - CARGA MANUAL (NICO)</t>
+          <t>REGISTRO DE GASTOS</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1496,7 +1496,7 @@
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="28" t="inlineStr">
         <is>
-          <t>Esta hoja es de uso exclusivo de Nico: anotar aca cada gasto real a medida que ocurre en el viaje (Uber, comidas, compras, propinas, etc.). Es independiente de la Matriz Financiera (que refleja lo ya reservado/facturado). Los totales de abajo se recalculan solos con formulas.</t>
+          <t>Registro de gastos reales del viaje (Uber, comidas, compras, propinas, etc.), independiente de la Matriz Financiera (que refleja lo ya reservado/facturado). Nico le cuenta cada gasto a Claude por chat y esta hoja se actualiza sola - no hace falta cargar nada a mano aca. Los totales de abajo se recalculan solos con formulas.</t>
         </is>
       </c>
     </row>
@@ -1543,13 +1543,13 @@
           <t>A confirmar</t>
         </is>
       </c>
-      <c r="B5" s="31" t="n"/>
+      <c r="B5" s="31" t="inlineStr"/>
       <c r="C5" s="30" t="inlineStr">
         <is>
           <t>Sena de reserva (confirmar si es Universal 63W124U2 o Disney #43028783 - ambas por $200)</t>
         </is>
       </c>
-      <c r="D5" s="31" t="n"/>
+      <c r="D5" s="31" t="inlineStr"/>
       <c r="E5" s="30" t="inlineStr">
         <is>
           <t>Nicolas - Tarjeta credito Santander Rio</t>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>Cargado por Claude a pedido de Nico; confirmar fecha exacta y a que reserva corresponde.</t>
+          <t>Avisado por Nico por chat; falta confirmar fecha exacta y a que reserva corresponde.</t>
         </is>
       </c>
     </row>
@@ -1924,386 +1924,215 @@
       <c r="F45" s="32" t="n"/>
       <c r="G45" s="31" t="n"/>
     </row>
-    <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="33" t="n"/>
-      <c r="B46" s="33" t="n"/>
-      <c r="C46" s="33" t="n"/>
-      <c r="D46" s="33" t="n"/>
-      <c r="E46" s="33" t="n"/>
-      <c r="F46" s="34" t="n"/>
-      <c r="G46" s="33" t="n"/>
-    </row>
-    <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="31" t="n"/>
-      <c r="B47" s="31" t="n"/>
-      <c r="C47" s="31" t="n"/>
-      <c r="D47" s="31" t="n"/>
-      <c r="E47" s="31" t="n"/>
-      <c r="F47" s="32" t="n"/>
-      <c r="G47" s="31" t="n"/>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>RESUMEN AUTOMATICO (se calcula solo a medida que cargas filas arriba)</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n"/>
+      <c r="C47" s="5" t="n"/>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="5" t="n"/>
+      <c r="F47" s="5" t="n"/>
+      <c r="G47" s="5" t="n"/>
     </row>
     <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="33" t="n"/>
-      <c r="B48" s="33" t="n"/>
-      <c r="C48" s="33" t="n"/>
-      <c r="D48" s="33" t="n"/>
-      <c r="E48" s="33" t="n"/>
-      <c r="F48" s="34" t="n"/>
-      <c r="G48" s="33" t="n"/>
+      <c r="A48" s="35" t="inlineStr">
+        <is>
+          <t>Total Nucleo 1</t>
+        </is>
+      </c>
+      <c r="B48" s="20">
+        <f>SUMIF($D$5:$D$45,"Nucleo 1",$F$5:$F$45)</f>
+        <v/>
+      </c>
+      <c r="C48" s="36" t="n"/>
+      <c r="D48" s="36" t="n"/>
+      <c r="E48" s="36" t="n"/>
+      <c r="F48" s="36" t="n"/>
+      <c r="G48" s="36" t="n"/>
     </row>
     <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="31" t="n"/>
-      <c r="B49" s="31" t="n"/>
-      <c r="C49" s="31" t="n"/>
-      <c r="D49" s="31" t="n"/>
-      <c r="E49" s="31" t="n"/>
-      <c r="F49" s="32" t="n"/>
-      <c r="G49" s="31" t="n"/>
+      <c r="A49" s="35" t="inlineStr">
+        <is>
+          <t>Total Nucleo 2</t>
+        </is>
+      </c>
+      <c r="B49" s="20">
+        <f>SUMIF($D$5:$D$45,"Nucleo 2",$F$5:$F$45)</f>
+        <v/>
+      </c>
+      <c r="C49" s="36" t="n"/>
+      <c r="D49" s="36" t="n"/>
+      <c r="E49" s="36" t="n"/>
+      <c r="F49" s="36" t="n"/>
+      <c r="G49" s="36" t="n"/>
     </row>
     <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="33" t="n"/>
-      <c r="B50" s="33" t="n"/>
-      <c r="C50" s="33" t="n"/>
-      <c r="D50" s="33" t="n"/>
-      <c r="E50" s="33" t="n"/>
-      <c r="F50" s="34" t="n"/>
-      <c r="G50" s="33" t="n"/>
+      <c r="A50" s="35" t="inlineStr">
+        <is>
+          <t>Total Nucleo 3</t>
+        </is>
+      </c>
+      <c r="B50" s="20">
+        <f>SUMIF($D$5:$D$45,"Nucleo 3",$F$5:$F$45)</f>
+        <v/>
+      </c>
+      <c r="C50" s="36" t="n"/>
+      <c r="D50" s="36" t="n"/>
+      <c r="E50" s="36" t="n"/>
+      <c r="F50" s="36" t="n"/>
+      <c r="G50" s="36" t="n"/>
     </row>
     <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="31" t="n"/>
-      <c r="B51" s="31" t="n"/>
-      <c r="C51" s="31" t="n"/>
-      <c r="D51" s="31" t="n"/>
-      <c r="E51" s="31" t="n"/>
-      <c r="F51" s="32" t="n"/>
-      <c r="G51" s="31" t="n"/>
+      <c r="A51" s="35" t="inlineStr">
+        <is>
+          <t>Total Compartido/Todos</t>
+        </is>
+      </c>
+      <c r="B51" s="20">
+        <f>SUMIF($D$5:$D$45,"Compartido/Todos",$F$5:$F$45)</f>
+        <v/>
+      </c>
+      <c r="C51" s="36" t="n"/>
+      <c r="D51" s="36" t="n"/>
+      <c r="E51" s="36" t="n"/>
+      <c r="F51" s="36" t="n"/>
+      <c r="G51" s="36" t="n"/>
     </row>
     <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="33" t="n"/>
-      <c r="B52" s="33" t="n"/>
-      <c r="C52" s="33" t="n"/>
-      <c r="D52" s="33" t="n"/>
-      <c r="E52" s="33" t="n"/>
-      <c r="F52" s="34" t="n"/>
-      <c r="G52" s="33" t="n"/>
-    </row>
-    <row r="53" ht="16" customHeight="1">
-      <c r="A53" s="31" t="n"/>
-      <c r="B53" s="31" t="n"/>
-      <c r="C53" s="31" t="n"/>
-      <c r="D53" s="31" t="n"/>
-      <c r="E53" s="31" t="n"/>
-      <c r="F53" s="32" t="n"/>
-      <c r="G53" s="31" t="n"/>
-    </row>
-    <row r="54" ht="16" customHeight="1">
-      <c r="A54" s="33" t="n"/>
-      <c r="B54" s="33" t="n"/>
-      <c r="C54" s="33" t="n"/>
-      <c r="D54" s="33" t="n"/>
-      <c r="E54" s="33" t="n"/>
-      <c r="F54" s="34" t="n"/>
-      <c r="G54" s="33" t="n"/>
-    </row>
-    <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="31" t="n"/>
-      <c r="B55" s="31" t="n"/>
-      <c r="C55" s="31" t="n"/>
-      <c r="D55" s="31" t="n"/>
-      <c r="E55" s="31" t="n"/>
-      <c r="F55" s="32" t="n"/>
-      <c r="G55" s="31" t="n"/>
-    </row>
-    <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="33" t="n"/>
-      <c r="B56" s="33" t="n"/>
-      <c r="C56" s="33" t="n"/>
-      <c r="D56" s="33" t="n"/>
-      <c r="E56" s="33" t="n"/>
-      <c r="F56" s="34" t="n"/>
-      <c r="G56" s="33" t="n"/>
-    </row>
-    <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="31" t="n"/>
-      <c r="B57" s="31" t="n"/>
-      <c r="C57" s="31" t="n"/>
-      <c r="D57" s="31" t="n"/>
-      <c r="E57" s="31" t="n"/>
-      <c r="F57" s="32" t="n"/>
-      <c r="G57" s="31" t="n"/>
-    </row>
-    <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="33" t="n"/>
-      <c r="B58" s="33" t="n"/>
-      <c r="C58" s="33" t="n"/>
-      <c r="D58" s="33" t="n"/>
-      <c r="E58" s="33" t="n"/>
-      <c r="F58" s="34" t="n"/>
-      <c r="G58" s="33" t="n"/>
-    </row>
-    <row r="59" ht="16" customHeight="1">
-      <c r="A59" s="31" t="n"/>
-      <c r="B59" s="31" t="n"/>
-      <c r="C59" s="31" t="n"/>
-      <c r="D59" s="31" t="n"/>
-      <c r="E59" s="31" t="n"/>
-      <c r="F59" s="32" t="n"/>
-      <c r="G59" s="31" t="n"/>
-    </row>
-    <row r="60" ht="16" customHeight="1">
-      <c r="A60" s="33" t="n"/>
-      <c r="B60" s="33" t="n"/>
-      <c r="C60" s="33" t="n"/>
-      <c r="D60" s="33" t="n"/>
-      <c r="E60" s="33" t="n"/>
-      <c r="F60" s="34" t="n"/>
-      <c r="G60" s="33" t="n"/>
-    </row>
-    <row r="61" ht="16" customHeight="1">
-      <c r="A61" s="31" t="n"/>
-      <c r="B61" s="31" t="n"/>
-      <c r="C61" s="31" t="n"/>
-      <c r="D61" s="31" t="n"/>
-      <c r="E61" s="31" t="n"/>
-      <c r="F61" s="32" t="n"/>
-      <c r="G61" s="31" t="n"/>
-    </row>
-    <row r="62" ht="16" customHeight="1">
-      <c r="A62" s="33" t="n"/>
-      <c r="B62" s="33" t="n"/>
-      <c r="C62" s="33" t="n"/>
-      <c r="D62" s="33" t="n"/>
-      <c r="E62" s="33" t="n"/>
-      <c r="F62" s="34" t="n"/>
-      <c r="G62" s="33" t="n"/>
-    </row>
-    <row r="63" ht="16" customHeight="1">
-      <c r="A63" s="31" t="n"/>
-      <c r="B63" s="31" t="n"/>
-      <c r="C63" s="31" t="n"/>
-      <c r="D63" s="31" t="n"/>
-      <c r="E63" s="31" t="n"/>
-      <c r="F63" s="32" t="n"/>
-      <c r="G63" s="31" t="n"/>
-    </row>
-    <row r="64" ht="16" customHeight="1">
-      <c r="A64" s="33" t="n"/>
-      <c r="B64" s="33" t="n"/>
-      <c r="C64" s="33" t="n"/>
-      <c r="D64" s="33" t="n"/>
-      <c r="E64" s="33" t="n"/>
-      <c r="F64" s="34" t="n"/>
-      <c r="G64" s="33" t="n"/>
-    </row>
-    <row r="66" ht="20" customHeight="1">
-      <c r="A66" s="4" t="inlineStr">
-        <is>
-          <t>RESUMEN AUTOMATICO (se calcula solo a medida que cargas filas arriba)</t>
-        </is>
-      </c>
-      <c r="B66" s="5" t="n"/>
-      <c r="C66" s="5" t="n"/>
-      <c r="D66" s="5" t="n"/>
-      <c r="E66" s="5" t="n"/>
-      <c r="F66" s="5" t="n"/>
-      <c r="G66" s="5" t="n"/>
-    </row>
-    <row r="67" ht="16" customHeight="1">
-      <c r="A67" s="35" t="inlineStr">
-        <is>
-          <t>Total Nucleo 1</t>
-        </is>
-      </c>
-      <c r="B67" s="20">
-        <f>SUMIF($D$5:$D$64,"Nucleo 1",$F$5:$F$64)</f>
-        <v/>
-      </c>
-      <c r="C67" s="36" t="n"/>
-      <c r="D67" s="36" t="n"/>
-      <c r="E67" s="36" t="n"/>
-      <c r="F67" s="36" t="n"/>
-      <c r="G67" s="36" t="n"/>
-    </row>
-    <row r="68" ht="16" customHeight="1">
-      <c r="A68" s="35" t="inlineStr">
-        <is>
-          <t>Total Nucleo 2</t>
-        </is>
-      </c>
-      <c r="B68" s="20">
-        <f>SUMIF($D$5:$D$64,"Nucleo 2",$F$5:$F$64)</f>
-        <v/>
-      </c>
-      <c r="C68" s="36" t="n"/>
-      <c r="D68" s="36" t="n"/>
-      <c r="E68" s="36" t="n"/>
-      <c r="F68" s="36" t="n"/>
-      <c r="G68" s="36" t="n"/>
-    </row>
-    <row r="69" ht="16" customHeight="1">
-      <c r="A69" s="35" t="inlineStr">
-        <is>
-          <t>Total Nucleo 3</t>
-        </is>
-      </c>
-      <c r="B69" s="20">
-        <f>SUMIF($D$5:$D$64,"Nucleo 3",$F$5:$F$64)</f>
-        <v/>
-      </c>
-      <c r="C69" s="36" t="n"/>
-      <c r="D69" s="36" t="n"/>
-      <c r="E69" s="36" t="n"/>
-      <c r="F69" s="36" t="n"/>
-      <c r="G69" s="36" t="n"/>
-    </row>
-    <row r="70" ht="16" customHeight="1">
-      <c r="A70" s="35" t="inlineStr">
-        <is>
-          <t>Total Compartido/Todos</t>
-        </is>
-      </c>
-      <c r="B70" s="20">
-        <f>SUMIF($D$5:$D$64,"Compartido/Todos",$F$5:$F$64)</f>
-        <v/>
-      </c>
-      <c r="C70" s="36" t="n"/>
-      <c r="D70" s="36" t="n"/>
-      <c r="E70" s="36" t="n"/>
-      <c r="F70" s="36" t="n"/>
-      <c r="G70" s="36" t="n"/>
-    </row>
-    <row r="71" ht="16" customHeight="1">
-      <c r="A71" s="35" t="inlineStr">
+      <c r="A52" s="35" t="inlineStr">
         <is>
           <t>Costo Nico (50% Nucleo 3)</t>
         </is>
       </c>
-      <c r="B71" s="20">
-        <f>B69/2</f>
-        <v/>
-      </c>
-      <c r="C71" s="36" t="n"/>
-      <c r="D71" s="36" t="n"/>
-      <c r="E71" s="36" t="n"/>
-      <c r="F71" s="36" t="n"/>
-      <c r="G71" s="36" t="n"/>
-    </row>
-    <row r="72" ht="20" customHeight="1">
-      <c r="A72" s="24" t="inlineStr">
+      <c r="B52" s="20">
+        <f>B50/2</f>
+        <v/>
+      </c>
+      <c r="C52" s="36" t="n"/>
+      <c r="D52" s="36" t="n"/>
+      <c r="E52" s="36" t="n"/>
+      <c r="F52" s="36" t="n"/>
+      <c r="G52" s="36" t="n"/>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="24" t="inlineStr">
         <is>
           <t>TOTAL REGISTRADO</t>
         </is>
       </c>
-      <c r="B72" s="26">
-        <f>SUM($F$5:$F$64)</f>
-        <v/>
-      </c>
-      <c r="C72" s="25" t="n"/>
-      <c r="D72" s="25" t="n"/>
-      <c r="E72" s="25" t="n"/>
-      <c r="F72" s="25" t="n"/>
-      <c r="G72" s="25" t="n"/>
-    </row>
-    <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="4" t="inlineStr">
+      <c r="B53" s="26">
+        <f>SUM($F$5:$F$45)</f>
+        <v/>
+      </c>
+      <c r="C53" s="25" t="n"/>
+      <c r="D53" s="25" t="n"/>
+      <c r="E53" s="25" t="n"/>
+      <c r="F53" s="25" t="n"/>
+      <c r="G53" s="25" t="n"/>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>DEUDAS ENTRE PERSONAS (adelantos de un integrante a nombre de otros)</t>
         </is>
       </c>
-      <c r="B75" s="5" t="n"/>
-      <c r="C75" s="5" t="n"/>
-      <c r="D75" s="5" t="n"/>
-      <c r="E75" s="5" t="n"/>
-      <c r="F75" s="5" t="n"/>
-      <c r="G75" s="5" t="n"/>
-    </row>
-    <row r="76" ht="18" customHeight="1">
-      <c r="A76" s="29" t="inlineStr">
+      <c r="B56" s="5" t="n"/>
+      <c r="C56" s="5" t="n"/>
+      <c r="D56" s="5" t="n"/>
+      <c r="E56" s="5" t="n"/>
+      <c r="F56" s="5" t="n"/>
+      <c r="G56" s="5" t="n"/>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="29" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B76" s="29" t="inlineStr">
+      <c r="B57" s="29" t="inlineStr">
         <is>
           <t>Adelanto pagado por</t>
         </is>
       </c>
-      <c r="C76" s="29" t="inlineStr">
+      <c r="C57" s="29" t="inlineStr">
         <is>
           <t>A cargo de</t>
         </is>
       </c>
-      <c r="D76" s="29" t="inlineStr">
+      <c r="D57" s="29" t="inlineStr">
         <is>
           <t>Monto USD</t>
         </is>
       </c>
-      <c r="E76" s="29" t="inlineStr">
+      <c r="E57" s="29" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F76" s="37" t="n"/>
-      <c r="G76" s="38" t="n"/>
-    </row>
-    <row r="77" ht="40" customHeight="1">
-      <c r="A77" s="19" t="inlineStr">
+      <c r="F57" s="37" t="n"/>
+      <c r="G57" s="38" t="n"/>
+    </row>
+    <row r="58" ht="40" customHeight="1">
+      <c r="A58" s="19" t="inlineStr">
         <is>
           <t>Universal Dockside (reserva conjunta 63W124U2: Florencia, German, Natalia, Nicolas)</t>
         </is>
       </c>
-      <c r="B77" s="19" t="inlineStr">
+      <c r="B58" s="19" t="inlineStr">
         <is>
           <t>German Agullo (pago la reserva completa)</t>
         </is>
       </c>
-      <c r="C77" s="19" t="inlineStr">
+      <c r="C58" s="19" t="inlineStr">
         <is>
           <t>Nicolas y Natalia (Nucleo 3) le deben a German la mitad de esta reserva + lo que falte pagar</t>
         </is>
       </c>
-      <c r="D77" s="20">
+      <c r="D58" s="20">
         <f>'Matriz Financiera'!F6</f>
         <v/>
       </c>
-      <c r="E77" s="39" t="inlineStr">
+      <c r="E58" s="39" t="inlineStr">
         <is>
           <t>Pendiente de liquidar con German</t>
         </is>
       </c>
-      <c r="F77" s="36" t="n"/>
-      <c r="G77" s="36" t="n"/>
-    </row>
-    <row r="78" ht="40" customHeight="1">
-      <c r="A78" s="19" t="inlineStr">
+      <c r="F58" s="36" t="n"/>
+      <c r="G58" s="36" t="n"/>
+    </row>
+    <row r="59" ht="40" customHeight="1">
+      <c r="A59" s="19" t="inlineStr">
         <is>
           <t>Disney Art of Animation (reserva #43028783: Natalia, Nicolas)</t>
         </is>
       </c>
-      <c r="B78" s="19" t="inlineStr">
+      <c r="B59" s="19" t="inlineStr">
         <is>
           <t>Nicolas y Natalia (pagan directo, sin intermediario)</t>
         </is>
       </c>
-      <c r="C78" s="19" t="inlineStr">
+      <c r="C59" s="19" t="inlineStr">
         <is>
           <t>N/A - no genera deuda entre personas</t>
         </is>
       </c>
-      <c r="D78" s="20">
+      <c r="D59" s="20">
         <f>'Matriz Financiera'!F5</f>
         <v/>
       </c>
-      <c r="E78" s="39" t="inlineStr">
+      <c r="E59" s="39" t="inlineStr">
         <is>
           <t>Gestionado directamente por Nucleo 3</t>
         </is>
       </c>
-      <c r="F78" s="36" t="n"/>
-      <c r="G78" s="36" t="n"/>
-    </row>
-    <row r="80" ht="30" customHeight="1">
-      <c r="A80" s="40" t="inlineStr">
+      <c r="F59" s="36" t="n"/>
+      <c r="G59" s="36" t="n"/>
+    </row>
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="40" t="inlineStr">
         <is>
           <t>El monto de la fila Universal esta enlazado por formula a la Matriz Financiera (Nucleo 3 = mitad de la reserva conjunta 63W124U2). Incluye la sena ya pagada y el saldo que falte liquidar con German a medida que se vaya pagando la reserva completa.</t>
         </is>
@@ -2311,20 +2140,20 @@
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="E77:G77"/>
-    <mergeCell ref="A66:G66"/>
+    <mergeCell ref="A61:G61"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A80:G80"/>
-    <mergeCell ref="E78:G78"/>
+    <mergeCell ref="A56:G56"/>
+    <mergeCell ref="E57:G57"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="E76:G76"/>
-    <mergeCell ref="A75:G75"/>
+    <mergeCell ref="E58:G58"/>
+    <mergeCell ref="E59:G59"/>
+    <mergeCell ref="A47:G47"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="B5:B64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B5:B45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Vuelos,Disney,Universal,Hospedaje Miami,Auto/Transporte,Comida,Compras,Seguro,Propinas,Otro"</formula1>
     </dataValidation>
-    <dataValidation sqref="D5:D64" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Nucleo 1,Nucleo 2,Nucleo 3,Compartido/Todos"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Registrar pago a Rodolfo por Hospedaje Miami y carpeta de comprobantes
Nico adelanto USD 1000 a Rodolfo, quien ya pago el total del alquiler
del departamento en Hollywood Beach. Se agrega el gasto real al
registro y una fila de deuda (Rodolfo -> Nucleo 2 + Nucleo 3) enlazada
por formula a la Matriz Financiera, a la espera del costo total del
alquiler para que se calcule solo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019LrLKneXbkjTi7bzStorH9
</commit_message>
<xml_diff>
--- a/Presupuesto_Florida_2027_Nico.xlsx
+++ b/Presupuesto_Florida_2027_Nico.xlsx
@@ -444,7 +444,7 @@
     </comment>
     <comment ref="B10" authorId="0" shapeId="0">
       <text>
-        <t>A COMPLETAR: no se encontro reserva en Drive. Cargar el costo total cuando se confirme el alojamiento.</t>
+        <t>A COMPLETAR: Rodolfo ya pago el total del alquiler. Cargar aca ese monto total cuando se confirme, para que se calcule la parte de cada nucleo (ver fila Rodolfo en Deudas Entre Personas, hoja Registro de Gastos).</t>
       </text>
     </comment>
     <comment ref="B11" authorId="0" shapeId="0">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Departamento 3/4 habitaciones, 17 al 22-feb-2027 (5 noches). Aun sin reservar.</t>
+          <t>Departamento 3/4 habitaciones, 17 al 22-feb-2027 (5 noches). Rodolfo pago el alquiler completo por adelantado.</t>
         </is>
       </c>
       <c r="C10" s="22" t="n">
@@ -1468,7 +1468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1565,13 +1565,39 @@
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="33" t="n"/>
-      <c r="B6" s="33" t="n"/>
-      <c r="C6" s="33" t="n"/>
-      <c r="D6" s="33" t="n"/>
-      <c r="E6" s="33" t="n"/>
-      <c r="F6" s="34" t="n"/>
-      <c r="G6" s="33" t="n"/>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>27-jul-2026</t>
+        </is>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>Hospedaje Miami</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>Pago a Rodolfo por el alquiler del departamento en Miami (Hollywood Beach) - Rodolfo pago el total del alquiler</t>
+        </is>
+      </c>
+      <c r="D6" s="33" t="inlineStr">
+        <is>
+          <t>Nucleo 3</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>Nicolas</t>
+        </is>
+      </c>
+      <c r="F6" s="34" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>Falta el costo TOTAL del alquiler (avisado por Nico) para calcular la parte proporcional exacta de cada nucleo en la Matriz Financiera.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="31" t="n"/>
@@ -1924,43 +1950,36 @@
       <c r="F45" s="32" t="n"/>
       <c r="G45" s="31" t="n"/>
     </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="4" t="inlineStr">
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="33" t="n"/>
+      <c r="B46" s="33" t="n"/>
+      <c r="C46" s="33" t="n"/>
+      <c r="D46" s="33" t="n"/>
+      <c r="E46" s="33" t="n"/>
+      <c r="F46" s="34" t="n"/>
+      <c r="G46" s="33" t="n"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>RESUMEN AUTOMATICO (se calcula solo a medida que cargas filas arriba)</t>
         </is>
       </c>
-      <c r="B47" s="5" t="n"/>
-      <c r="C47" s="5" t="n"/>
-      <c r="D47" s="5" t="n"/>
-      <c r="E47" s="5" t="n"/>
-      <c r="F47" s="5" t="n"/>
-      <c r="G47" s="5" t="n"/>
-    </row>
-    <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="35" t="inlineStr">
-        <is>
-          <t>Total Nucleo 1</t>
-        </is>
-      </c>
-      <c r="B48" s="20">
-        <f>SUMIF($D$5:$D$45,"Nucleo 1",$F$5:$F$45)</f>
-        <v/>
-      </c>
-      <c r="C48" s="36" t="n"/>
-      <c r="D48" s="36" t="n"/>
-      <c r="E48" s="36" t="n"/>
-      <c r="F48" s="36" t="n"/>
-      <c r="G48" s="36" t="n"/>
+      <c r="B48" s="5" t="n"/>
+      <c r="C48" s="5" t="n"/>
+      <c r="D48" s="5" t="n"/>
+      <c r="E48" s="5" t="n"/>
+      <c r="F48" s="5" t="n"/>
+      <c r="G48" s="5" t="n"/>
     </row>
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="35" t="inlineStr">
         <is>
-          <t>Total Nucleo 2</t>
+          <t>Total Nucleo 1</t>
         </is>
       </c>
       <c r="B49" s="20">
-        <f>SUMIF($D$5:$D$45,"Nucleo 2",$F$5:$F$45)</f>
+        <f>SUMIF($D$5:$D$46,"Nucleo 1",$F$5:$F$46)</f>
         <v/>
       </c>
       <c r="C49" s="36" t="n"/>
@@ -1972,11 +1991,11 @@
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="35" t="inlineStr">
         <is>
-          <t>Total Nucleo 3</t>
+          <t>Total Nucleo 2</t>
         </is>
       </c>
       <c r="B50" s="20">
-        <f>SUMIF($D$5:$D$45,"Nucleo 3",$F$5:$F$45)</f>
+        <f>SUMIF($D$5:$D$46,"Nucleo 2",$F$5:$F$46)</f>
         <v/>
       </c>
       <c r="C50" s="36" t="n"/>
@@ -1988,11 +2007,11 @@
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="35" t="inlineStr">
         <is>
-          <t>Total Compartido/Todos</t>
+          <t>Total Nucleo 3</t>
         </is>
       </c>
       <c r="B51" s="20">
-        <f>SUMIF($D$5:$D$45,"Compartido/Todos",$F$5:$F$45)</f>
+        <f>SUMIF($D$5:$D$46,"Nucleo 3",$F$5:$F$46)</f>
         <v/>
       </c>
       <c r="C51" s="36" t="n"/>
@@ -2004,11 +2023,11 @@
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="35" t="inlineStr">
         <is>
-          <t>Costo Nico (50% Nucleo 3)</t>
+          <t>Total Compartido/Todos</t>
         </is>
       </c>
       <c r="B52" s="20">
-        <f>B50/2</f>
+        <f>SUMIF($D$5:$D$46,"Compartido/Todos",$F$5:$F$46)</f>
         <v/>
       </c>
       <c r="C52" s="36" t="n"/>
@@ -2017,143 +2036,188 @@
       <c r="F52" s="36" t="n"/>
       <c r="G52" s="36" t="n"/>
     </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="24" t="inlineStr">
+    <row r="53" ht="16" customHeight="1">
+      <c r="A53" s="35" t="inlineStr">
+        <is>
+          <t>Costo Nico (50% Nucleo 3)</t>
+        </is>
+      </c>
+      <c r="B53" s="20">
+        <f>B51/2</f>
+        <v/>
+      </c>
+      <c r="C53" s="36" t="n"/>
+      <c r="D53" s="36" t="n"/>
+      <c r="E53" s="36" t="n"/>
+      <c r="F53" s="36" t="n"/>
+      <c r="G53" s="36" t="n"/>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="24" t="inlineStr">
         <is>
           <t>TOTAL REGISTRADO</t>
         </is>
       </c>
-      <c r="B53" s="26">
-        <f>SUM($F$5:$F$45)</f>
-        <v/>
-      </c>
-      <c r="C53" s="25" t="n"/>
-      <c r="D53" s="25" t="n"/>
-      <c r="E53" s="25" t="n"/>
-      <c r="F53" s="25" t="n"/>
-      <c r="G53" s="25" t="n"/>
-    </row>
-    <row r="56" ht="20" customHeight="1">
-      <c r="A56" s="4" t="inlineStr">
+      <c r="B54" s="26">
+        <f>SUM($F$5:$F$46)</f>
+        <v/>
+      </c>
+      <c r="C54" s="25" t="n"/>
+      <c r="D54" s="25" t="n"/>
+      <c r="E54" s="25" t="n"/>
+      <c r="F54" s="25" t="n"/>
+      <c r="G54" s="25" t="n"/>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>DEUDAS ENTRE PERSONAS (adelantos de un integrante a nombre de otros)</t>
         </is>
       </c>
-      <c r="B56" s="5" t="n"/>
-      <c r="C56" s="5" t="n"/>
-      <c r="D56" s="5" t="n"/>
-      <c r="E56" s="5" t="n"/>
-      <c r="F56" s="5" t="n"/>
-      <c r="G56" s="5" t="n"/>
-    </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="29" t="inlineStr">
+      <c r="B57" s="5" t="n"/>
+      <c r="C57" s="5" t="n"/>
+      <c r="D57" s="5" t="n"/>
+      <c r="E57" s="5" t="n"/>
+      <c r="F57" s="5" t="n"/>
+      <c r="G57" s="5" t="n"/>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="29" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B57" s="29" t="inlineStr">
+      <c r="B58" s="29" t="inlineStr">
         <is>
           <t>Adelanto pagado por</t>
         </is>
       </c>
-      <c r="C57" s="29" t="inlineStr">
+      <c r="C58" s="29" t="inlineStr">
         <is>
           <t>A cargo de</t>
         </is>
       </c>
-      <c r="D57" s="29" t="inlineStr">
+      <c r="D58" s="29" t="inlineStr">
         <is>
           <t>Monto USD</t>
         </is>
       </c>
-      <c r="E57" s="29" t="inlineStr">
+      <c r="E58" s="29" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F57" s="37" t="n"/>
-      <c r="G57" s="38" t="n"/>
-    </row>
-    <row r="58" ht="40" customHeight="1">
-      <c r="A58" s="19" t="inlineStr">
-        <is>
-          <t>Universal Dockside (reserva conjunta 63W124U2: Florencia, German, Natalia, Nicolas)</t>
-        </is>
-      </c>
-      <c r="B58" s="19" t="inlineStr">
-        <is>
-          <t>German Agullo (pago la reserva completa)</t>
-        </is>
-      </c>
-      <c r="C58" s="19" t="inlineStr">
-        <is>
-          <t>Nicolas y Natalia (Nucleo 3) le deben a German la mitad de esta reserva + lo que falte pagar</t>
-        </is>
-      </c>
-      <c r="D58" s="20">
-        <f>'Matriz Financiera'!F6</f>
-        <v/>
-      </c>
-      <c r="E58" s="39" t="inlineStr">
-        <is>
-          <t>Pendiente de liquidar con German</t>
-        </is>
-      </c>
-      <c r="F58" s="36" t="n"/>
-      <c r="G58" s="36" t="n"/>
+      <c r="F58" s="37" t="n"/>
+      <c r="G58" s="38" t="n"/>
     </row>
     <row r="59" ht="40" customHeight="1">
       <c r="A59" s="19" t="inlineStr">
         <is>
-          <t>Disney Art of Animation (reserva #43028783: Natalia, Nicolas)</t>
+          <t>Hospedaje Miami (departamento Hollywood Beach, 17 al 22-feb)</t>
         </is>
       </c>
       <c r="B59" s="19" t="inlineStr">
         <is>
-          <t>Nicolas y Natalia (pagan directo, sin intermediario)</t>
+          <t>Rodolfo Agullo (pago el total del alquiler por adelantado)</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>N/A - no genera deuda entre personas</t>
+          <t>Florencia y German (Nucleo 2) + Natalia y Nicolas (Nucleo 3), cada uno su parte proporcional</t>
         </is>
       </c>
       <c r="D59" s="20">
-        <f>'Matriz Financiera'!F5</f>
+        <f>'Matriz Financiera'!E10+'Matriz Financiera'!F10</f>
         <v/>
       </c>
       <c r="E59" s="39" t="inlineStr">
         <is>
-          <t>Gestionado directamente por Nucleo 3</t>
+          <t>Pendiente: falta cargar el costo TOTAL del alquiler en la Matriz Financiera (fila Hospedaje Miami) para que este monto se calcule solo. Nico ya le adelanto $1000 a Rodolfo a cuenta de esto (ver arriba).</t>
         </is>
       </c>
       <c r="F59" s="36" t="n"/>
       <c r="G59" s="36" t="n"/>
     </row>
-    <row r="61" ht="30" customHeight="1">
-      <c r="A61" s="40" t="inlineStr">
+    <row r="60" ht="40" customHeight="1">
+      <c r="A60" s="19" t="inlineStr">
+        <is>
+          <t>Universal Dockside (reserva conjunta 63W124U2: Florencia, German, Natalia, Nicolas)</t>
+        </is>
+      </c>
+      <c r="B60" s="19" t="inlineStr">
+        <is>
+          <t>German Agullo (pago la reserva completa)</t>
+        </is>
+      </c>
+      <c r="C60" s="19" t="inlineStr">
+        <is>
+          <t>Nicolas y Natalia (Nucleo 3) le deben a German la mitad de esta reserva + lo que falte pagar</t>
+        </is>
+      </c>
+      <c r="D60" s="20">
+        <f>'Matriz Financiera'!F6</f>
+        <v/>
+      </c>
+      <c r="E60" s="39" t="inlineStr">
+        <is>
+          <t>Pendiente de liquidar con German</t>
+        </is>
+      </c>
+      <c r="F60" s="36" t="n"/>
+      <c r="G60" s="36" t="n"/>
+    </row>
+    <row r="61" ht="40" customHeight="1">
+      <c r="A61" s="19" t="inlineStr">
+        <is>
+          <t>Disney Art of Animation (reserva #43028783: Natalia, Nicolas)</t>
+        </is>
+      </c>
+      <c r="B61" s="19" t="inlineStr">
+        <is>
+          <t>Nicolas y Natalia (pagan directo, sin intermediario)</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>N/A - no genera deuda entre personas</t>
+        </is>
+      </c>
+      <c r="D61" s="20">
+        <f>'Matriz Financiera'!F5</f>
+        <v/>
+      </c>
+      <c r="E61" s="39" t="inlineStr">
+        <is>
+          <t>Gestionado directamente por Nucleo 3</t>
+        </is>
+      </c>
+      <c r="F61" s="36" t="n"/>
+      <c r="G61" s="36" t="n"/>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="40" t="inlineStr">
         <is>
           <t>El monto de la fila Universal esta enlazado por formula a la Matriz Financiera (Nucleo 3 = mitad de la reserva conjunta 63W124U2). Incluye la sena ya pagada y el saldo que falte liquidar con German a medida que se vaya pagando la reserva completa.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A61:G61"/>
+  <mergeCells count="9">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A56:G56"/>
-    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="E60:G60"/>
+    <mergeCell ref="A63:G63"/>
+    <mergeCell ref="E61:G61"/>
+    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="E58:G58"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="E58:G58"/>
+    <mergeCell ref="A57:G57"/>
     <mergeCell ref="E59:G59"/>
-    <mergeCell ref="A47:G47"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="B5:B45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B5:B46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Vuelos,Disney,Universal,Hospedaje Miami,Auto/Transporte,Comida,Compras,Seguro,Propinas,Otro"</formula1>
     </dataValidation>
-    <dataValidation sqref="D5:D45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Nucleo 1,Nucleo 2,Nucleo 3,Compartido/Todos"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Cargar monto real de Hospedaje Miami desde el comprobante en Drive
Factura #648 (Hyde Beach House Apt 3708, Hollywood Beach): estadia
$3,250 + limpieza final $270 = $3,520 total, pagado por adelantado por
Rodolfo. Se actualiza la Matriz Financiera con el monto real (deja de
ser estimacion) y se ajusta la fila de deuda pendiente con Rodolfo:
Nucleo 3 ya salda su parte con el pago de $1,000 de Nico, solo queda
pendiente la parte de Florencia/German.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019LrLKneXbkjTi7bzStorH9
</commit_message>
<xml_diff>
--- a/Presupuesto_Florida_2027_Nico.xlsx
+++ b/Presupuesto_Florida_2027_Nico.xlsx
@@ -444,7 +444,7 @@
     </comment>
     <comment ref="B10" authorId="0" shapeId="0">
       <text>
-        <t>A COMPLETAR: Rodolfo ya pago el total del alquiler. Cargar aca ese monto total cuando se confirme, para que se calcule la parte de cada nucleo (ver fila Rodolfo en Deudas Entre Personas, hoja Registro de Gastos).</t>
+        <t>Monto real segun factura #648 (comprobante en Drive, carpeta Reservas hospedajes). Reparto proporcional por PAX: N1 incluye a Delfina. Nicolas ya le pago a Rodolfo $1,000 a cuenta de la parte de Nucleo 3 (ver Registro de Gastos); puede quedar un saldo menor si no coincide exacto con F10/2 de esta fila.</t>
       </text>
     </comment>
     <comment ref="B11" authorId="0" shapeId="0">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>Departamento 3/4 habitaciones, 17 al 22-feb-2027 (5 noches). Rodolfo pago el alquiler completo por adelantado.</t>
-        </is>
-      </c>
-      <c r="C10" s="22" t="n">
-        <v>0</v>
+          <t>Hyde Beach House Apt 3708 (3 dormitorios), 4010 South Ocean Drive, Hollywood Beach FL 33019. Confirmacion #593958171. Check-in 17-feb-2027 16:00, check-out 22-feb-2027 11:00. Incluye parking y servicio de playa para 2 personas ($300 de garantia con tarjeta al check-in). Factura #648: estadia $3,250.00 + limpieza final $270.00. Rodolfo pago el total por adelantado; la parte de Delfina la cubren Rodolfo y Claudia directamente dentro del Nucleo 1.</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="n">
+        <v>3520</v>
       </c>
       <c r="D10" s="21">
         <f>$C10*N1_PAX/TOTAL_PAX</f>
@@ -1577,7 +1577,7 @@
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>Pago a Rodolfo por el alquiler del departamento en Miami (Hollywood Beach) - Rodolfo pago el total del alquiler</t>
+          <t>Pago a Rodolfo por el alquiler del departamento en Miami (Hyde Beach House Apt 3708, factura #648: $3,520.00 - comprobante en Drive). Cubre aproximadamente la parte de Nucleo 3 (Natalia y Nicolas).</t>
         </is>
       </c>
       <c r="D6" s="33" t="inlineStr">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="G6" s="19" t="inlineStr">
         <is>
-          <t>Falta el costo TOTAL del alquiler (avisado por Nico) para calcular la parte proporcional exacta de cada nucleo en la Matriz Financiera.</t>
+          <t>Parte de Nucleo 3 es $1,005.71 exacto ($3,520/7 x 2); Nicolas pago $1,000, puede quedar un saldo menor de $5.71 con Rodolfo. La parte de Delfina la cubren Rodolfo y Claudia directo. Falta que Florencia y German le paguen a Rodolfo su parte (~$1,005.71).</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2113,7 @@
     <row r="59" ht="40" customHeight="1">
       <c r="A59" s="19" t="inlineStr">
         <is>
-          <t>Hospedaje Miami (departamento Hollywood Beach, 17 al 22-feb)</t>
+          <t>Hyde Beach House Apt 3708 - Hospedaje Miami (factura #648: $3,520) - SALDO PENDIENTE</t>
         </is>
       </c>
       <c r="B59" s="19" t="inlineStr">
@@ -2123,16 +2123,16 @@
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Florencia y German (Nucleo 2) + Natalia y Nicolas (Nucleo 3), cada uno su parte proporcional</t>
+          <t>Florencia y German (Nucleo 2)</t>
         </is>
       </c>
       <c r="D59" s="20">
-        <f>'Matriz Financiera'!E10+'Matriz Financiera'!F10</f>
+        <f>'Matriz Financiera'!E10</f>
         <v/>
       </c>
       <c r="E59" s="39" t="inlineStr">
         <is>
-          <t>Pendiente: falta cargar el costo TOTAL del alquiler en la Matriz Financiera (fila Hospedaje Miami) para que este monto se calcule solo. Nico ya le adelanto $1000 a Rodolfo a cuenta de esto (ver arriba).</t>
+          <t>Pendiente de liquidar con Rodolfo. Nucleo 3 (Natalia y Nicolas) YA PAGO $1,000 a cuenta (ver Registro de Gastos arriba; su parte exacta figura en la fila Hospedaje Miami de la Matriz Financiera, puede quedar un saldo chico). Nucleo 1 no debe nada porque cubre su propia parte, incluida la de Delfina.</t>
         </is>
       </c>
       <c r="F59" s="36" t="n"/>

</xml_diff>

<commit_message>
Confirmar sena de $200 como pago de Disney (Nucleo 3)
Nico confirmo que la sena de $200 pagada con Santander Rio corresponde
a la reserva Disney #43028783 (Natalia y Nicolas), no a Universal.
Todavia no hay pagos propios en la reserva Universal (la esta cubriendo
German).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019LrLKneXbkjTi7bzStorH9
</commit_message>
<xml_diff>
--- a/Presupuesto_Florida_2027_Nico.xlsx
+++ b/Presupuesto_Florida_2027_Nico.xlsx
@@ -1540,16 +1540,24 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="30" t="inlineStr">
         <is>
-          <t>A confirmar</t>
-        </is>
-      </c>
-      <c r="B5" s="31" t="inlineStr"/>
+          <t>09-jul-2026</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="inlineStr">
+        <is>
+          <t>Disney</t>
+        </is>
+      </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>Sena de reserva (confirmar si es Universal 63W124U2 o Disney #43028783 - ambas por $200)</t>
-        </is>
-      </c>
-      <c r="D5" s="31" t="inlineStr"/>
+          <t>Sena de la reserva Disney Art of Animation #43028783 (Natalia y Nicolas, Nucleo 3)</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>Nucleo 3</t>
+        </is>
+      </c>
       <c r="E5" s="30" t="inlineStr">
         <is>
           <t>Nicolas - Tarjeta credito Santander Rio</t>
@@ -1560,7 +1568,7 @@
       </c>
       <c r="G5" s="30" t="inlineStr">
         <is>
-          <t>Avisado por Nico por chat; falta confirmar fecha exacta y a que reserva corresponde.</t>
+          <t>Confirmado por Nico: la sena de $200 fue para Disney, no para Universal. Todavia no pago nada de la reserva Universal (la esta pagando German).</t>
         </is>
       </c>
     </row>

</xml_diff>